<commit_message>
completed HITL fuzzy match for 2024
</commit_message>
<xml_diff>
--- a/assetManagement/reportOuts/fuzzyMatches_HITL_20241003.xlsx
+++ b/assetManagement/reportOuts/fuzzyMatches_HITL_20241003.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joeduprey/repos/metadataVerification/assetManagement/reportOuts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C14B2D0C-908B-3A4D-9587-E0AC6E8C1045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BD7F846A-0BB6-9440-AD85-89B87356E59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37520" yWindow="-10580" windowWidth="35220" windowHeight="19140" xr2:uid="{D3F55A4A-1B46-8740-A2A9-3D1205BC3408}"/>
+    <workbookView xWindow="140" yWindow="760" windowWidth="33120" windowHeight="19740" xr2:uid="{D3F55A4A-1B46-8740-A2A9-3D1205BC3408}"/>
   </bookViews>
   <sheets>
     <sheet name="fuzzyMatches_HITL_20241003" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="1397" uniqueCount="984">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="1432" uniqueCount="1017">
   <si>
     <t>referenceDesignator</t>
   </si>
@@ -2097,9 +2097,6 @@
     <t>Z:\For_Science\Mitch\Equipment_photos\LJ01A\OPTAAC103_2023\OPTAAC103_20230816_222607_predeploy.JPG</t>
   </si>
   <si>
-    <t>05-08317</t>
-  </si>
-  <si>
     <t>Z:\For_Science\Mitch\Equipment_photos\LJ01A\CTDPFB101_2023\CTDPFB101_20230816_222713_predeploy.JPG,Z:\For_Science\Mitch\Equipment_photos\LJ01A\CTDPFB101_2023\CTDPFB101_20230816_222746_predeploy.JPG,Z:\For_Science\Mitch\Equipment_photos\LJ01A\CTDPFB101_2023\CTDPFB101_20230817_111018_predeploy.JPG</t>
   </si>
   <si>
@@ -2934,18 +2931,6 @@
     <t>IMG_1545.JPG</t>
   </si>
   <si>
-    <t>potential typo in image asset id</t>
-  </si>
-  <si>
-    <t>need to look at image</t>
-  </si>
-  <si>
-    <t>head, hardware TODO</t>
-  </si>
-  <si>
-    <t>TODO</t>
-  </si>
-  <si>
     <t>[ 'ATAPL-70114-00006']</t>
   </si>
   <si>
@@ -2976,7 +2961,121 @@
     <t>Head</t>
   </si>
   <si>
-    <t xml:space="preserve">SN confusion 05 or 1273	</t>
+    <t xml:space="preserve">typo in physical SN, I think it should be ATAPL-58334-00004	 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">physical SN fragment 1179-7232, probably ATAPL-66662-00003	</t>
+  </si>
+  <si>
+    <t>ATAPL-58694-00002</t>
+  </si>
+  <si>
+    <t>ATAPL-58694-00002 found in image upon review</t>
+  </si>
+  <si>
+    <t>ATAPL-67627-00001</t>
+  </si>
+  <si>
+    <t>ATAPL-67627-00001 found in image upon review</t>
+  </si>
+  <si>
+    <t>ATAPL-58324-00005 found in image</t>
+  </si>
+  <si>
+    <t>ATAPL-58324-00005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATAPL-66943-00002 found in image typo? should be ATAPL-69943-00002 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATAPL-67627-00004 found in image </t>
+  </si>
+  <si>
+    <t>matches DOSTAD - not sure why script missed this</t>
+  </si>
+  <si>
+    <t>ATAPL-68020-00007 matches 618, not sure why script missed</t>
+  </si>
+  <si>
+    <t>ATAPL-78520-00004</t>
+  </si>
+  <si>
+    <t>ATAPL-78520-00004 found in image</t>
+  </si>
+  <si>
+    <t>Equipment_Photos/VISIONS24/PC03A/PC03A_2024/VADCPB301_2024/VADCPB301_20240811_110122_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>no SN in image</t>
+  </si>
+  <si>
+    <t>no SN for CAMHD, wrong part SN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no SN for CAMDS, need to look at image, ATAPL-78437-00010	</t>
+  </si>
+  <si>
+    <t>no SN for CAMDS, typo on physical SN missing 0</t>
+  </si>
+  <si>
+    <t>head, hardware</t>
+  </si>
+  <si>
+    <t>no SN for CAMDS, Missing 0? Should be ATAPL-78437-00012?</t>
+  </si>
+  <si>
+    <t>no SN for CAMDS, camera case as image SN? Should be ATAPL-78437-00011?</t>
+  </si>
+  <si>
+    <t>no SN for CAMDS, serial number in two images should be ATAPL-78437-00001</t>
+  </si>
+  <si>
+    <t>no SN for CAMDS, ATAPL-78438-00012 in image probably ATAPL-78438-00012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no SN for CAMDS, likely ATAPL-78437-00006, parts confusion? </t>
+  </si>
+  <si>
+    <t>image SN not available</t>
+  </si>
+  <si>
+    <t>['ATOSU-67977-00007	']</t>
+  </si>
+  <si>
+    <t>ATOSU-67977-00007 per SN on raw data archive</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no SN available for CAMHD, 70502 SN found in image, matches HD cam part</t>
+  </si>
+  <si>
+    <t>['ATAPL-58334-00004']</t>
+  </si>
+  <si>
+    <t>['ATOSU-63259-00003']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">should be ATOSU-63259-00003	</t>
+  </si>
+  <si>
+    <t>['ATAPL-58694-00002']</t>
+  </si>
+  <si>
+    <t>['ATAPL-67627-00001']</t>
+  </si>
+  <si>
+    <t>['ATAPL-58324-00005']</t>
+  </si>
+  <si>
+    <t>['ATAPL-66943-00002']</t>
+  </si>
+  <si>
+    <t>['ATAPL-67627-00004']</t>
+  </si>
+  <si>
+    <t>['ATAPL-68020-00007 ']</t>
+  </si>
+  <si>
+    <t>['ATAPL-78520-00004']</t>
   </si>
 </sst>
 </file>
@@ -3307,19 +3406,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FFC00000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3491,8 +3590,8 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3872,7 +3971,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="3" max="3" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" customWidth="1"/>
+    <col min="4" max="4" width="171.33203125" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="23.6640625" customWidth="1"/>
     <col min="7" max="7" width="39" customWidth="1"/>
@@ -3881,7 +3981,7 @@
     <col min="10" max="10" width="18.33203125" customWidth="1"/>
     <col min="11" max="11" width="13.83203125" customWidth="1"/>
     <col min="12" max="12" width="17.33203125" customWidth="1"/>
-    <col min="13" max="13" width="19" customWidth="1"/>
+    <col min="13" max="13" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -4091,8 +4191,8 @@
       <c r="F7" t="s">
         <v>36</v>
       </c>
-      <c r="M7" t="s">
-        <v>969</v>
+      <c r="M7" s="4" t="s">
+        <v>994</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -4111,8 +4211,8 @@
       <c r="F8" t="s">
         <v>39</v>
       </c>
-      <c r="M8" t="s">
-        <v>970</v>
+      <c r="M8" s="4" t="s">
+        <v>995</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -4392,8 +4492,14 @@
       <c r="E17">
         <v>1233</v>
       </c>
-      <c r="M17" s="7" t="s">
-        <v>983</v>
+      <c r="G17" t="s">
+        <v>1008</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>1009</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.2">
@@ -4673,8 +4779,8 @@
       <c r="F26" t="s">
         <v>128</v>
       </c>
-      <c r="M26" t="s">
-        <v>970</v>
+      <c r="M26" s="4" t="s">
+        <v>996</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
@@ -5114,19 +5220,19 @@
         <v>200</v>
       </c>
       <c r="G40" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="H40" t="s">
         <v>201</v>
       </c>
       <c r="I40" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="L40" t="b">
         <v>1</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>971</v>
+        <v>997</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.2">
@@ -5406,6 +5512,9 @@
       <c r="F49" t="s">
         <v>243</v>
       </c>
+      <c r="M49" s="4" t="s">
+        <v>998</v>
+      </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50">
@@ -5553,19 +5662,19 @@
         <v>266</v>
       </c>
       <c r="G54" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="H54" t="s">
         <v>571</v>
       </c>
       <c r="I54" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="L54" t="b">
         <v>1</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>977</v>
+        <v>972</v>
       </c>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.2">
@@ -5782,8 +5891,14 @@
       <c r="F61" t="s">
         <v>302</v>
       </c>
-      <c r="M61" s="4" t="s">
-        <v>972</v>
+      <c r="G61" t="s">
+        <v>1007</v>
+      </c>
+      <c r="L61" t="b">
+        <v>1</v>
+      </c>
+      <c r="M61" s="5" t="s">
+        <v>978</v>
       </c>
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.2">
@@ -5862,6 +5977,9 @@
       <c r="F64" t="s">
         <v>313</v>
       </c>
+      <c r="M64" s="4" t="s">
+        <v>999</v>
+      </c>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A65">
@@ -6250,7 +6368,7 @@
       </c>
       <c r="M76" s="3"/>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>75</v>
       </c>
@@ -6265,6 +6383,9 @@
       </c>
       <c r="F77" t="s">
         <v>375</v>
+      </c>
+      <c r="M77" s="4" t="s">
+        <v>1000</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.2">
@@ -6343,6 +6464,9 @@
       <c r="E80">
         <v>1794559</v>
       </c>
+      <c r="M80" s="6" t="s">
+        <v>1003</v>
+      </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A81">
@@ -6426,6 +6550,18 @@
       <c r="E83" t="s">
         <v>400</v>
       </c>
+      <c r="F83" t="s">
+        <v>840</v>
+      </c>
+      <c r="G83" t="s">
+        <v>841</v>
+      </c>
+      <c r="L83" t="b">
+        <v>1</v>
+      </c>
+      <c r="M83" s="5" t="s">
+        <v>979</v>
+      </c>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A84">
@@ -6443,6 +6579,18 @@
       <c r="E84">
         <v>1794924</v>
       </c>
+      <c r="F84" t="s">
+        <v>980</v>
+      </c>
+      <c r="G84" t="s">
+        <v>1010</v>
+      </c>
+      <c r="L84" t="b">
+        <v>1</v>
+      </c>
+      <c r="M84" s="5" t="s">
+        <v>981</v>
+      </c>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A85">
@@ -6658,6 +6806,18 @@
       <c r="E91">
         <v>2595170</v>
       </c>
+      <c r="F91" t="s">
+        <v>982</v>
+      </c>
+      <c r="G91" t="s">
+        <v>1011</v>
+      </c>
+      <c r="L91" t="b">
+        <v>1</v>
+      </c>
+      <c r="M91" s="5" t="s">
+        <v>983</v>
+      </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A92">
@@ -7347,6 +7507,9 @@
       <c r="F113" t="s">
         <v>525</v>
       </c>
+      <c r="M113" s="4" t="s">
+        <v>1001</v>
+      </c>
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A114">
@@ -7523,6 +7686,9 @@
       <c r="F119" t="s">
         <v>547</v>
       </c>
+      <c r="M119" s="7" t="s">
+        <v>1003</v>
+      </c>
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A120">
@@ -7930,8 +8096,20 @@
       <c r="D132" t="s">
         <v>605</v>
       </c>
+      <c r="E132">
+        <v>138</v>
+      </c>
       <c r="F132" t="s">
         <v>606</v>
+      </c>
+      <c r="G132" t="s">
+        <v>1004</v>
+      </c>
+      <c r="L132" t="b">
+        <v>1</v>
+      </c>
+      <c r="M132" s="5" t="s">
+        <v>1005</v>
       </c>
     </row>
     <row r="133" spans="1:13" x14ac:dyDescent="0.2">
@@ -8476,16 +8654,16 @@
         <v>675</v>
       </c>
       <c r="G149" t="s">
+        <v>911</v>
+      </c>
+      <c r="I149" t="s">
         <v>912</v>
       </c>
-      <c r="I149" t="s">
-        <v>913</v>
-      </c>
       <c r="L149" t="b">
         <v>1</v>
       </c>
-      <c r="M149" s="6" t="s">
-        <v>978</v>
+      <c r="M149" s="5" t="s">
+        <v>973</v>
       </c>
     </row>
     <row r="150" spans="1:13" x14ac:dyDescent="0.2">
@@ -8570,6 +8748,18 @@
       <c r="E152" t="s">
         <v>687</v>
       </c>
+      <c r="F152" t="s">
+        <v>985</v>
+      </c>
+      <c r="G152" t="s">
+        <v>1012</v>
+      </c>
+      <c r="L152" t="b">
+        <v>1</v>
+      </c>
+      <c r="M152" s="5" t="s">
+        <v>984</v>
+      </c>
     </row>
     <row r="153" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A153">
@@ -8614,8 +8804,17 @@
       <c r="D154" t="s">
         <v>689</v>
       </c>
-      <c r="E154" t="s">
-        <v>690</v>
+      <c r="E154">
+        <v>155</v>
+      </c>
+      <c r="G154" t="s">
+        <v>1013</v>
+      </c>
+      <c r="L154" t="b">
+        <v>1</v>
+      </c>
+      <c r="M154" s="5" t="s">
+        <v>986</v>
       </c>
     </row>
     <row r="155" spans="1:13" x14ac:dyDescent="0.2">
@@ -8629,10 +8828,22 @@
         <v>2023</v>
       </c>
       <c r="D155" t="s">
+        <v>690</v>
+      </c>
+      <c r="E155" t="s">
         <v>691</v>
       </c>
-      <c r="E155" t="s">
-        <v>692</v>
+      <c r="F155" t="s">
+        <v>691</v>
+      </c>
+      <c r="G155" t="s">
+        <v>1014</v>
+      </c>
+      <c r="L155" t="b">
+        <v>1</v>
+      </c>
+      <c r="M155" s="5" t="s">
+        <v>987</v>
       </c>
     </row>
     <row r="156" spans="1:13" x14ac:dyDescent="0.2">
@@ -8646,10 +8857,19 @@
         <v>2023</v>
       </c>
       <c r="D156" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="E156" t="s">
         <v>32</v>
+      </c>
+      <c r="G156" t="s">
+        <v>33</v>
+      </c>
+      <c r="L156" t="b">
+        <v>1</v>
+      </c>
+      <c r="M156" s="5" t="s">
+        <v>988</v>
       </c>
     </row>
     <row r="157" spans="1:13" x14ac:dyDescent="0.2">
@@ -8663,13 +8883,13 @@
         <v>2023</v>
       </c>
       <c r="D157" t="s">
+        <v>693</v>
+      </c>
+      <c r="E157">
+        <v>1</v>
+      </c>
+      <c r="F157" t="s">
         <v>694</v>
-      </c>
-      <c r="E157">
-        <v>1</v>
-      </c>
-      <c r="F157" t="s">
-        <v>695</v>
       </c>
       <c r="G157" t="s">
         <v>309</v>
@@ -8696,7 +8916,7 @@
         <v>2023</v>
       </c>
       <c r="D158" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="E158">
         <v>2</v>
@@ -8726,7 +8946,7 @@
         <v>2023</v>
       </c>
       <c r="D159" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="E159">
         <v>3</v>
@@ -8756,16 +8976,16 @@
         <v>2023</v>
       </c>
       <c r="D160" t="s">
+        <v>697</v>
+      </c>
+      <c r="E160" t="s">
         <v>698</v>
       </c>
-      <c r="E160" t="s">
+      <c r="F160" t="s">
         <v>699</v>
       </c>
-      <c r="F160" t="s">
+      <c r="G160" t="s">
         <v>700</v>
-      </c>
-      <c r="G160" t="s">
-        <v>701</v>
       </c>
       <c r="K160" t="b">
         <v>1</v>
@@ -8786,16 +9006,16 @@
         <v>2023</v>
       </c>
       <c r="D161" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E161">
         <v>18975</v>
       </c>
       <c r="G161" t="s">
+        <v>702</v>
+      </c>
+      <c r="I161" t="s">
         <v>703</v>
-      </c>
-      <c r="I161" t="s">
-        <v>704</v>
       </c>
       <c r="J161" t="b">
         <v>1</v>
@@ -8816,16 +9036,16 @@
         <v>2023</v>
       </c>
       <c r="D162" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="E162">
         <v>4</v>
       </c>
       <c r="G162" t="s">
+        <v>705</v>
+      </c>
+      <c r="I162" t="s">
         <v>706</v>
-      </c>
-      <c r="I162" t="s">
-        <v>707</v>
       </c>
       <c r="J162" t="b">
         <v>1</v>
@@ -8840,25 +9060,25 @@
         <v>161</v>
       </c>
       <c r="B163" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="C163">
         <v>2023</v>
       </c>
       <c r="D163" t="s">
+        <v>708</v>
+      </c>
+      <c r="E163" t="s">
         <v>709</v>
       </c>
-      <c r="E163" t="s">
+      <c r="F163" t="s">
         <v>710</v>
       </c>
-      <c r="F163" t="s">
+      <c r="G163" t="s">
         <v>711</v>
       </c>
-      <c r="G163" t="s">
+      <c r="I163" t="s">
         <v>712</v>
-      </c>
-      <c r="I163" t="s">
-        <v>713</v>
       </c>
       <c r="J163" t="b">
         <v>1</v>
@@ -8879,13 +9099,16 @@
         <v>2023</v>
       </c>
       <c r="D164" t="s">
+        <v>713</v>
+      </c>
+      <c r="E164" t="s">
         <v>714</v>
       </c>
-      <c r="E164" t="s">
+      <c r="F164" t="s">
         <v>715</v>
       </c>
-      <c r="F164" t="s">
-        <v>716</v>
+      <c r="M164" s="4" t="s">
+        <v>1006</v>
       </c>
     </row>
     <row r="165" spans="1:13" x14ac:dyDescent="0.2">
@@ -8899,22 +9122,22 @@
         <v>2023</v>
       </c>
       <c r="D165" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="E165">
         <v>307</v>
       </c>
       <c r="G165" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="I165" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="L165" t="b">
         <v>1</v>
       </c>
       <c r="M165" s="5" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
     </row>
     <row r="166" spans="1:13" x14ac:dyDescent="0.2">
@@ -8928,13 +9151,13 @@
         <v>2023</v>
       </c>
       <c r="D166" t="s">
+        <v>717</v>
+      </c>
+      <c r="F166" t="s">
         <v>718</v>
       </c>
-      <c r="F166" t="s">
+      <c r="G166" t="s">
         <v>719</v>
-      </c>
-      <c r="G166" t="s">
-        <v>720</v>
       </c>
       <c r="K166" t="b">
         <v>1</v>
@@ -8955,13 +9178,13 @@
         <v>2023</v>
       </c>
       <c r="D167" t="s">
+        <v>720</v>
+      </c>
+      <c r="F167" t="s">
         <v>721</v>
       </c>
-      <c r="F167" t="s">
+      <c r="G167" t="s">
         <v>722</v>
-      </c>
-      <c r="G167" t="s">
-        <v>723</v>
       </c>
       <c r="K167" t="b">
         <v>1</v>
@@ -8982,13 +9205,13 @@
         <v>2023</v>
       </c>
       <c r="D168" t="s">
+        <v>723</v>
+      </c>
+      <c r="F168" t="s">
         <v>724</v>
       </c>
-      <c r="F168" t="s">
+      <c r="G168" t="s">
         <v>725</v>
-      </c>
-      <c r="G168" t="s">
-        <v>726</v>
       </c>
       <c r="K168" t="b">
         <v>1</v>
@@ -9009,19 +9232,19 @@
         <v>2023</v>
       </c>
       <c r="D169" t="s">
+        <v>726</v>
+      </c>
+      <c r="E169" t="s">
         <v>727</v>
       </c>
-      <c r="E169" t="s">
+      <c r="F169" t="s">
         <v>728</v>
       </c>
-      <c r="F169" t="s">
+      <c r="G169" t="s">
         <v>729</v>
       </c>
-      <c r="G169" t="s">
+      <c r="I169" t="s">
         <v>730</v>
-      </c>
-      <c r="I169" t="s">
-        <v>731</v>
       </c>
       <c r="J169" t="b">
         <v>1</v>
@@ -9042,13 +9265,13 @@
         <v>2023</v>
       </c>
       <c r="D170" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="E170">
         <v>1130</v>
       </c>
       <c r="F170" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="G170" t="s">
         <v>276</v>
@@ -9075,19 +9298,19 @@
         <v>2023</v>
       </c>
       <c r="D171" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E171">
         <v>3716</v>
       </c>
       <c r="F171" t="s">
+        <v>734</v>
+      </c>
+      <c r="G171" t="s">
         <v>735</v>
       </c>
-      <c r="G171" t="s">
+      <c r="I171" t="s">
         <v>736</v>
-      </c>
-      <c r="I171" t="s">
-        <v>737</v>
       </c>
       <c r="J171" t="b">
         <v>1</v>
@@ -9108,19 +9331,19 @@
         <v>2023</v>
       </c>
       <c r="D172" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="E172">
         <v>3637</v>
       </c>
       <c r="F172" t="s">
+        <v>738</v>
+      </c>
+      <c r="G172" t="s">
         <v>739</v>
       </c>
-      <c r="G172" t="s">
+      <c r="I172" t="s">
         <v>740</v>
-      </c>
-      <c r="I172" t="s">
-        <v>741</v>
       </c>
       <c r="J172" t="b">
         <v>1</v>
@@ -9141,13 +9364,13 @@
         <v>2023</v>
       </c>
       <c r="D173" t="s">
+        <v>741</v>
+      </c>
+      <c r="F173" t="s">
         <v>742</v>
       </c>
-      <c r="F173" t="s">
+      <c r="G173" t="s">
         <v>743</v>
-      </c>
-      <c r="G173" t="s">
-        <v>744</v>
       </c>
       <c r="K173" t="b">
         <v>1</v>
@@ -9168,19 +9391,19 @@
         <v>2023</v>
       </c>
       <c r="D174" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E174">
         <v>18974</v>
       </c>
       <c r="F174" t="s">
+        <v>745</v>
+      </c>
+      <c r="G174" t="s">
         <v>746</v>
       </c>
-      <c r="G174" t="s">
+      <c r="I174" t="s">
         <v>747</v>
-      </c>
-      <c r="I174" t="s">
-        <v>748</v>
       </c>
       <c r="J174" t="b">
         <v>1</v>
@@ -9201,22 +9424,22 @@
         <v>2023</v>
       </c>
       <c r="D175" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E175">
         <v>61247</v>
       </c>
       <c r="F175" t="s">
+        <v>749</v>
+      </c>
+      <c r="G175" t="s">
         <v>750</v>
       </c>
-      <c r="G175" t="s">
+      <c r="H175" t="s">
         <v>751</v>
       </c>
-      <c r="H175" t="s">
+      <c r="I175" t="s">
         <v>752</v>
-      </c>
-      <c r="I175" t="s">
-        <v>753</v>
       </c>
       <c r="L175" t="b">
         <v>1</v>
@@ -9234,22 +9457,22 @@
         <v>2023</v>
       </c>
       <c r="D176" t="s">
+        <v>753</v>
+      </c>
+      <c r="E176" t="s">
         <v>754</v>
       </c>
-      <c r="E176" t="s">
+      <c r="F176" t="s">
         <v>755</v>
       </c>
-      <c r="F176" t="s">
+      <c r="G176" t="s">
         <v>756</v>
-      </c>
-      <c r="G176" t="s">
-        <v>757</v>
       </c>
       <c r="H176" t="s">
         <v>505</v>
       </c>
       <c r="I176" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="L176" t="b">
         <v>1</v>
@@ -9267,16 +9490,16 @@
         <v>2023</v>
       </c>
       <c r="D177" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E177">
         <v>1362</v>
       </c>
       <c r="G177" t="s">
+        <v>759</v>
+      </c>
+      <c r="I177" t="s">
         <v>760</v>
-      </c>
-      <c r="I177" t="s">
-        <v>761</v>
       </c>
       <c r="J177" t="b">
         <v>1</v>
@@ -9297,16 +9520,16 @@
         <v>2023</v>
       </c>
       <c r="D178" t="s">
+        <v>761</v>
+      </c>
+      <c r="E178" t="s">
         <v>762</v>
       </c>
-      <c r="E178" t="s">
+      <c r="G178" t="s">
         <v>763</v>
       </c>
-      <c r="G178" t="s">
+      <c r="I178" t="s">
         <v>764</v>
-      </c>
-      <c r="I178" t="s">
-        <v>765</v>
       </c>
       <c r="J178" t="b">
         <v>1</v>
@@ -9327,19 +9550,19 @@
         <v>2023</v>
       </c>
       <c r="D179" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="E179">
         <v>473</v>
       </c>
       <c r="F179" t="s">
+        <v>766</v>
+      </c>
+      <c r="G179" t="s">
         <v>767</v>
       </c>
-      <c r="G179" t="s">
+      <c r="I179" t="s">
         <v>768</v>
-      </c>
-      <c r="I179" t="s">
-        <v>769</v>
       </c>
       <c r="J179" t="b">
         <v>1</v>
@@ -9360,19 +9583,19 @@
         <v>2023</v>
       </c>
       <c r="D180" t="s">
+        <v>769</v>
+      </c>
+      <c r="E180" t="s">
         <v>770</v>
       </c>
-      <c r="E180" t="s">
+      <c r="F180" t="s">
         <v>771</v>
       </c>
-      <c r="F180" t="s">
+      <c r="G180" t="s">
         <v>772</v>
       </c>
-      <c r="G180" t="s">
+      <c r="I180" t="s">
         <v>773</v>
-      </c>
-      <c r="I180" t="s">
-        <v>774</v>
       </c>
       <c r="J180" t="b">
         <v>1</v>
@@ -9393,19 +9616,19 @@
         <v>2023</v>
       </c>
       <c r="D181" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E181">
         <v>1294</v>
       </c>
       <c r="F181" t="s">
+        <v>775</v>
+      </c>
+      <c r="G181" t="s">
         <v>776</v>
       </c>
-      <c r="G181" t="s">
+      <c r="I181" t="s">
         <v>777</v>
-      </c>
-      <c r="I181" t="s">
-        <v>778</v>
       </c>
       <c r="J181" t="b">
         <v>1</v>
@@ -9426,19 +9649,19 @@
         <v>2023</v>
       </c>
       <c r="D182" t="s">
+        <v>778</v>
+      </c>
+      <c r="E182" t="s">
         <v>779</v>
       </c>
-      <c r="E182" t="s">
+      <c r="F182" t="s">
         <v>780</v>
       </c>
-      <c r="F182" t="s">
+      <c r="G182" t="s">
         <v>781</v>
       </c>
-      <c r="G182" t="s">
+      <c r="I182" t="s">
         <v>782</v>
-      </c>
-      <c r="I182" t="s">
-        <v>783</v>
       </c>
       <c r="J182" t="b">
         <v>1</v>
@@ -9459,19 +9682,19 @@
         <v>2023</v>
       </c>
       <c r="D183" t="s">
+        <v>783</v>
+      </c>
+      <c r="E183" t="s">
         <v>784</v>
       </c>
-      <c r="E183" t="s">
+      <c r="F183" t="s">
         <v>785</v>
       </c>
-      <c r="F183" t="s">
+      <c r="G183" t="s">
         <v>786</v>
       </c>
-      <c r="G183" t="s">
+      <c r="I183" t="s">
         <v>787</v>
-      </c>
-      <c r="I183" t="s">
-        <v>788</v>
       </c>
       <c r="J183" t="b">
         <v>1</v>
@@ -9492,16 +9715,16 @@
         <v>2023</v>
       </c>
       <c r="D184" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="E184">
         <v>1293</v>
       </c>
       <c r="G184" t="s">
+        <v>789</v>
+      </c>
+      <c r="I184" t="s">
         <v>790</v>
-      </c>
-      <c r="I184" t="s">
-        <v>791</v>
       </c>
       <c r="J184" t="b">
         <v>1</v>
@@ -9522,16 +9745,16 @@
         <v>2023</v>
       </c>
       <c r="D185" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="E185">
         <v>251</v>
       </c>
       <c r="G185" t="s">
+        <v>792</v>
+      </c>
+      <c r="I185" t="s">
         <v>793</v>
-      </c>
-      <c r="I185" t="s">
-        <v>794</v>
       </c>
       <c r="J185" t="b">
         <v>1</v>
@@ -9546,22 +9769,22 @@
         <v>184</v>
       </c>
       <c r="B186" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="C186">
         <v>2023</v>
       </c>
       <c r="D186" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="E186">
         <v>1402</v>
       </c>
       <c r="G186" t="s">
+        <v>796</v>
+      </c>
+      <c r="I186" t="s">
         <v>797</v>
-      </c>
-      <c r="I186" t="s">
-        <v>798</v>
       </c>
       <c r="J186" t="b">
         <v>1</v>
@@ -9576,25 +9799,25 @@
         <v>185</v>
       </c>
       <c r="B187" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="C187">
         <v>2023</v>
       </c>
       <c r="D187" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="E187">
         <v>293</v>
       </c>
       <c r="F187" t="s">
+        <v>800</v>
+      </c>
+      <c r="G187" t="s">
         <v>801</v>
       </c>
-      <c r="G187" t="s">
+      <c r="I187" t="s">
         <v>802</v>
-      </c>
-      <c r="I187" t="s">
-        <v>803</v>
       </c>
       <c r="J187" t="b">
         <v>1</v>
@@ -9615,10 +9838,19 @@
         <v>2023</v>
       </c>
       <c r="D188" t="s">
+        <v>803</v>
+      </c>
+      <c r="E188" t="s">
         <v>804</v>
       </c>
-      <c r="E188" t="s">
-        <v>805</v>
+      <c r="G188" t="s">
+        <v>1015</v>
+      </c>
+      <c r="L188" t="b">
+        <v>1</v>
+      </c>
+      <c r="M188" s="5" t="s">
+        <v>989</v>
       </c>
     </row>
     <row r="189" spans="1:13" x14ac:dyDescent="0.2">
@@ -9632,22 +9864,22 @@
         <v>2023</v>
       </c>
       <c r="D189" t="s">
+        <v>805</v>
+      </c>
+      <c r="E189" t="s">
         <v>806</v>
       </c>
-      <c r="E189" t="s">
+      <c r="F189" t="s">
         <v>807</v>
       </c>
-      <c r="F189" t="s">
+      <c r="G189" t="s">
         <v>808</v>
-      </c>
-      <c r="G189" t="s">
-        <v>809</v>
       </c>
       <c r="H189" t="s">
         <v>598</v>
       </c>
       <c r="I189" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="L189" t="b">
         <v>1</v>
@@ -9665,19 +9897,19 @@
         <v>2023</v>
       </c>
       <c r="D190" t="s">
+        <v>810</v>
+      </c>
+      <c r="E190" t="s">
         <v>811</v>
       </c>
-      <c r="E190" t="s">
+      <c r="F190" t="s">
         <v>812</v>
       </c>
-      <c r="F190" t="s">
+      <c r="G190" t="s">
         <v>813</v>
       </c>
-      <c r="G190" t="s">
+      <c r="I190" t="s">
         <v>814</v>
-      </c>
-      <c r="I190" t="s">
-        <v>815</v>
       </c>
       <c r="J190" t="b">
         <v>1</v>
@@ -9698,19 +9930,19 @@
         <v>2023</v>
       </c>
       <c r="D191" t="s">
+        <v>815</v>
+      </c>
+      <c r="E191" t="s">
         <v>816</v>
       </c>
-      <c r="E191" t="s">
+      <c r="F191" t="s">
         <v>817</v>
       </c>
-      <c r="F191" t="s">
+      <c r="G191" t="s">
         <v>818</v>
       </c>
-      <c r="G191" t="s">
+      <c r="I191" t="s">
         <v>819</v>
-      </c>
-      <c r="I191" t="s">
-        <v>820</v>
       </c>
       <c r="J191" t="b">
         <v>1</v>
@@ -9731,19 +9963,19 @@
         <v>2023</v>
       </c>
       <c r="D192" t="s">
+        <v>820</v>
+      </c>
+      <c r="E192" t="s">
         <v>821</v>
       </c>
-      <c r="E192" t="s">
+      <c r="F192" t="s">
         <v>822</v>
       </c>
-      <c r="F192" t="s">
+      <c r="G192" t="s">
         <v>823</v>
       </c>
-      <c r="G192" t="s">
+      <c r="I192" t="s">
         <v>824</v>
-      </c>
-      <c r="I192" t="s">
-        <v>825</v>
       </c>
       <c r="J192" t="b">
         <v>1</v>
@@ -9764,13 +9996,16 @@
         <v>2023</v>
       </c>
       <c r="D193" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E193">
         <v>301</v>
       </c>
       <c r="F193" t="s">
-        <v>827</v>
+        <v>826</v>
+      </c>
+      <c r="M193" s="4" t="s">
+        <v>1002</v>
       </c>
     </row>
     <row r="194" spans="1:13" x14ac:dyDescent="0.2">
@@ -9784,13 +10019,13 @@
         <v>2023</v>
       </c>
       <c r="D194" t="s">
+        <v>827</v>
+      </c>
+      <c r="F194" t="s">
         <v>828</v>
       </c>
-      <c r="F194" t="s">
+      <c r="G194" t="s">
         <v>829</v>
-      </c>
-      <c r="G194" t="s">
-        <v>830</v>
       </c>
       <c r="K194" t="b">
         <v>1</v>
@@ -9811,16 +10046,16 @@
         <v>2023</v>
       </c>
       <c r="D195" t="s">
+        <v>830</v>
+      </c>
+      <c r="E195" t="s">
         <v>831</v>
-      </c>
-      <c r="E195" t="s">
-        <v>832</v>
       </c>
       <c r="G195" t="s">
         <v>447</v>
       </c>
       <c r="I195" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="J195" t="b">
         <v>1</v>
@@ -9835,13 +10070,13 @@
         <v>194</v>
       </c>
       <c r="B196" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C196">
         <v>2023</v>
       </c>
       <c r="D196" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E196">
         <v>2</v>
@@ -9865,13 +10100,13 @@
         <v>195</v>
       </c>
       <c r="B197" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C197">
         <v>2023</v>
       </c>
       <c r="D197" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="E197">
         <v>2</v>
@@ -9895,25 +10130,25 @@
         <v>196</v>
       </c>
       <c r="B198" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="C198">
         <v>2024</v>
       </c>
       <c r="D198" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E198">
         <v>1405</v>
       </c>
       <c r="F198" t="s">
+        <v>836</v>
+      </c>
+      <c r="G198" t="s">
         <v>837</v>
       </c>
-      <c r="G198" t="s">
+      <c r="I198" t="s">
         <v>838</v>
-      </c>
-      <c r="I198" t="s">
-        <v>839</v>
       </c>
       <c r="J198" t="b">
         <v>1</v>
@@ -9934,22 +10169,22 @@
         <v>2024</v>
       </c>
       <c r="D199" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="E199">
         <v>7232</v>
       </c>
       <c r="F199" t="s">
+        <v>840</v>
+      </c>
+      <c r="G199" t="s">
         <v>841</v>
-      </c>
-      <c r="G199" t="s">
-        <v>842</v>
       </c>
       <c r="H199" t="s">
         <v>495</v>
       </c>
       <c r="I199" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="L199" t="b">
         <v>1</v>
@@ -9961,13 +10196,25 @@
         <v>198</v>
       </c>
       <c r="B200" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="C200">
         <v>2024</v>
       </c>
-      <c r="M200" t="s">
-        <v>972</v>
+      <c r="D200" t="s">
+        <v>992</v>
+      </c>
+      <c r="F200" t="s">
+        <v>990</v>
+      </c>
+      <c r="G200" t="s">
+        <v>1016</v>
+      </c>
+      <c r="L200" t="b">
+        <v>1</v>
+      </c>
+      <c r="M200" s="5" t="s">
+        <v>991</v>
       </c>
     </row>
     <row r="201" spans="1:13" x14ac:dyDescent="0.2">
@@ -9981,10 +10228,10 @@
         <v>2024</v>
       </c>
       <c r="D201" t="s">
+        <v>844</v>
+      </c>
+      <c r="E201" t="s">
         <v>845</v>
-      </c>
-      <c r="E201" t="s">
-        <v>846</v>
       </c>
       <c r="F201" t="s">
         <v>330</v>
@@ -10005,22 +10252,22 @@
         <v>200</v>
       </c>
       <c r="B202" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="C202">
         <v>2024</v>
       </c>
       <c r="D202" t="s">
+        <v>847</v>
+      </c>
+      <c r="E202" t="s">
         <v>848</v>
       </c>
-      <c r="E202" t="s">
+      <c r="F202" t="s">
         <v>849</v>
       </c>
-      <c r="F202" t="s">
+      <c r="G202" t="s">
         <v>850</v>
-      </c>
-      <c r="G202" t="s">
-        <v>851</v>
       </c>
       <c r="K202" t="b">
         <v>1</v>
@@ -10035,25 +10282,25 @@
         <v>201</v>
       </c>
       <c r="B203" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="C203">
         <v>2024</v>
       </c>
       <c r="D203" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="E203">
         <v>1399</v>
       </c>
       <c r="F203" t="s">
+        <v>853</v>
+      </c>
+      <c r="G203" t="s">
         <v>854</v>
       </c>
-      <c r="G203" t="s">
+      <c r="I203" t="s">
         <v>855</v>
-      </c>
-      <c r="I203" t="s">
-        <v>856</v>
       </c>
       <c r="J203" t="b">
         <v>1</v>
@@ -10068,13 +10315,13 @@
         <v>202</v>
       </c>
       <c r="B204" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="C204">
         <v>2024</v>
       </c>
-      <c r="M204" t="s">
-        <v>972</v>
+      <c r="M204" s="6" t="s">
+        <v>993</v>
       </c>
     </row>
     <row r="205" spans="1:13" x14ac:dyDescent="0.2">
@@ -10082,25 +10329,25 @@
         <v>203</v>
       </c>
       <c r="B205" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="C205">
         <v>2024</v>
       </c>
       <c r="D205" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="E205">
         <v>1400</v>
       </c>
       <c r="F205" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="G205" t="s">
         <v>860</v>
       </c>
-      <c r="G205" t="s">
+      <c r="I205" t="s">
         <v>861</v>
-      </c>
-      <c r="I205" t="s">
-        <v>862</v>
       </c>
       <c r="J205" t="b">
         <v>1</v>
@@ -10121,7 +10368,7 @@
         <v>2020</v>
       </c>
       <c r="D206" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="E206">
         <v>19003</v>
@@ -10154,22 +10401,22 @@
         <v>2020</v>
       </c>
       <c r="D207" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="E207">
         <v>7230</v>
       </c>
       <c r="F207" t="s">
+        <v>864</v>
+      </c>
+      <c r="G207" t="s">
         <v>865</v>
-      </c>
-      <c r="G207" t="s">
-        <v>866</v>
       </c>
       <c r="H207" t="s">
         <v>495</v>
       </c>
       <c r="I207" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="L207" t="b">
         <v>1</v>
@@ -10187,7 +10434,7 @@
         <v>2020</v>
       </c>
       <c r="D208" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="E208">
         <v>216</v>
@@ -10220,7 +10467,7 @@
         <v>2020</v>
       </c>
       <c r="D209" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="E209" s="2">
         <v>50078167</v>
@@ -10253,7 +10500,7 @@
         <v>2020</v>
       </c>
       <c r="D210" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="E210">
         <v>169</v>
@@ -10286,7 +10533,7 @@
         <v>2020</v>
       </c>
       <c r="D211" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="E211" t="s">
         <v>70</v>
@@ -10319,7 +10566,7 @@
         <v>2020</v>
       </c>
       <c r="D212" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="E212" t="s">
         <v>76</v>
@@ -10352,7 +10599,7 @@
         <v>2020</v>
       </c>
       <c r="D213" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="E213">
         <v>21498</v>
@@ -10385,7 +10632,7 @@
         <v>2020</v>
       </c>
       <c r="D214" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="E214">
         <v>7231</v>
@@ -10418,7 +10665,7 @@
         <v>2020</v>
       </c>
       <c r="D215" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="E215">
         <v>133</v>
@@ -10451,10 +10698,10 @@
         <v>2020</v>
       </c>
       <c r="D216" t="s">
+        <v>874</v>
+      </c>
+      <c r="E216" t="s">
         <v>875</v>
-      </c>
-      <c r="E216" t="s">
-        <v>876</v>
       </c>
       <c r="F216" t="s">
         <v>104</v>
@@ -10463,7 +10710,7 @@
         <v>105</v>
       </c>
       <c r="I216" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="J216" t="b">
         <v>1</v>
@@ -10484,7 +10731,7 @@
         <v>2020</v>
       </c>
       <c r="D217" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="E217">
         <v>191</v>
@@ -10517,7 +10764,7 @@
         <v>2020</v>
       </c>
       <c r="D218" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="E218" t="s">
         <v>114</v>
@@ -10550,7 +10797,7 @@
         <v>2020</v>
       </c>
       <c r="D219" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="E219" t="s">
         <v>120</v>
@@ -10583,7 +10830,7 @@
         <v>2020</v>
       </c>
       <c r="D220" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="E220" t="s">
         <v>210</v>
@@ -10616,13 +10863,13 @@
         <v>2020</v>
       </c>
       <c r="D221" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="E221">
         <v>1131</v>
       </c>
       <c r="F221" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G221" t="s">
         <v>396</v>
@@ -10649,7 +10896,7 @@
         <v>2020</v>
       </c>
       <c r="D222" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="E222">
         <v>3400</v>
@@ -10682,19 +10929,19 @@
         <v>2020</v>
       </c>
       <c r="D223" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="E223">
         <v>3398</v>
       </c>
       <c r="F223" t="s">
+        <v>884</v>
+      </c>
+      <c r="G223" t="s">
         <v>885</v>
       </c>
-      <c r="G223" t="s">
+      <c r="I223" t="s">
         <v>886</v>
-      </c>
-      <c r="I223" t="s">
-        <v>887</v>
       </c>
       <c r="J223" t="b">
         <v>1</v>
@@ -10715,13 +10962,13 @@
         <v>2020</v>
       </c>
       <c r="D224" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="E224">
         <v>137</v>
       </c>
       <c r="F224" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="G224" t="s">
         <v>229</v>
@@ -10748,13 +10995,13 @@
         <v>2020</v>
       </c>
       <c r="D225" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="E225">
         <v>2</v>
       </c>
       <c r="F225" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="G225" t="s">
         <v>316</v>
@@ -10781,13 +11028,13 @@
         <v>2020</v>
       </c>
       <c r="D226" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E226">
         <v>50018</v>
       </c>
       <c r="F226" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="G226" t="s">
         <v>154</v>
@@ -10814,19 +11061,19 @@
         <v>2020</v>
       </c>
       <c r="D227" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="E227">
         <v>215</v>
       </c>
       <c r="F227" t="s">
+        <v>893</v>
+      </c>
+      <c r="G227" t="s">
         <v>894</v>
       </c>
-      <c r="G227" t="s">
+      <c r="I227" t="s">
         <v>895</v>
-      </c>
-      <c r="I227" t="s">
-        <v>896</v>
       </c>
       <c r="J227" t="b">
         <v>1</v>
@@ -10847,7 +11094,7 @@
         <v>2020</v>
       </c>
       <c r="D228" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="E228" t="s">
         <v>158</v>
@@ -10880,7 +11127,7 @@
         <v>2020</v>
       </c>
       <c r="D229" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="E229" t="s">
         <v>164</v>
@@ -10913,7 +11160,7 @@
         <v>2020</v>
       </c>
       <c r="D230" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="E230">
         <v>50019</v>
@@ -10946,7 +11193,7 @@
         <v>2020</v>
       </c>
       <c r="D231" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="E231" t="s">
         <v>480</v>
@@ -10979,7 +11226,7 @@
         <v>2020</v>
       </c>
       <c r="D232" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="E232">
         <v>1150</v>
@@ -11012,19 +11259,19 @@
         <v>2020</v>
       </c>
       <c r="D233" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="E233">
         <v>128</v>
       </c>
       <c r="F233" t="s">
+        <v>902</v>
+      </c>
+      <c r="G233" t="s">
         <v>903</v>
       </c>
-      <c r="G233" t="s">
+      <c r="I233" t="s">
         <v>904</v>
-      </c>
-      <c r="I233" t="s">
-        <v>905</v>
       </c>
       <c r="J233" t="b">
         <v>1</v>
@@ -11039,25 +11286,25 @@
         <v>28</v>
       </c>
       <c r="B234" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C234">
         <v>2020</v>
       </c>
       <c r="D234" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="E234">
         <v>267</v>
       </c>
       <c r="F234" t="s">
+        <v>907</v>
+      </c>
+      <c r="G234" t="s">
         <v>908</v>
       </c>
-      <c r="G234" t="s">
+      <c r="I234" t="s">
         <v>909</v>
-      </c>
-      <c r="I234" t="s">
-        <v>910</v>
       </c>
       <c r="J234" t="b">
         <v>1</v>
@@ -11078,7 +11325,7 @@
         <v>2020</v>
       </c>
       <c r="D235" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="E235">
         <v>344</v>
@@ -11087,10 +11334,10 @@
         <v>675</v>
       </c>
       <c r="G235" t="s">
+        <v>911</v>
+      </c>
+      <c r="I235" t="s">
         <v>912</v>
-      </c>
-      <c r="I235" t="s">
-        <v>913</v>
       </c>
       <c r="J235" t="b">
         <v>1</v>
@@ -11111,7 +11358,7 @@
         <v>2020</v>
       </c>
       <c r="D236" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E236" t="s">
         <v>475</v>
@@ -11144,19 +11391,19 @@
         <v>2020</v>
       </c>
       <c r="D237" t="s">
+        <v>914</v>
+      </c>
+      <c r="E237" t="s">
         <v>915</v>
       </c>
-      <c r="E237" t="s">
+      <c r="F237" t="s">
         <v>916</v>
       </c>
-      <c r="F237" t="s">
+      <c r="G237" t="s">
         <v>917</v>
       </c>
-      <c r="G237" t="s">
+      <c r="I237" t="s">
         <v>918</v>
-      </c>
-      <c r="I237" t="s">
-        <v>919</v>
       </c>
       <c r="J237" t="b">
         <v>1</v>
@@ -11177,7 +11424,7 @@
         <v>2020</v>
       </c>
       <c r="D238" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E238">
         <v>1214</v>
@@ -11210,7 +11457,7 @@
         <v>2020</v>
       </c>
       <c r="D239" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="E239">
         <v>3098</v>
@@ -11243,7 +11490,7 @@
         <v>2020</v>
       </c>
       <c r="D240" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E240">
         <v>3099</v>
@@ -11276,7 +11523,7 @@
         <v>2020</v>
       </c>
       <c r="D241" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="E241">
         <v>458</v>
@@ -11309,19 +11556,19 @@
         <v>2020</v>
       </c>
       <c r="D242" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="E242">
         <v>18478</v>
       </c>
       <c r="F242" t="s">
+        <v>924</v>
+      </c>
+      <c r="G242" t="s">
         <v>925</v>
       </c>
-      <c r="G242" t="s">
+      <c r="I242" t="s">
         <v>926</v>
-      </c>
-      <c r="I242" t="s">
-        <v>927</v>
       </c>
       <c r="J242" t="b">
         <v>1</v>
@@ -11342,7 +11589,7 @@
         <v>2020</v>
       </c>
       <c r="D243" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="E243">
         <v>19075</v>
@@ -11375,7 +11622,7 @@
         <v>2020</v>
       </c>
       <c r="D244" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="E244">
         <v>6914</v>
@@ -11408,19 +11655,19 @@
         <v>2020</v>
       </c>
       <c r="D245" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="E245">
         <v>275</v>
       </c>
       <c r="F245" t="s">
+        <v>929</v>
+      </c>
+      <c r="G245" t="s">
         <v>930</v>
       </c>
-      <c r="G245" t="s">
+      <c r="I245" t="s">
         <v>931</v>
-      </c>
-      <c r="I245" t="s">
-        <v>932</v>
       </c>
       <c r="J245" t="b">
         <v>1</v>
@@ -11441,7 +11688,7 @@
         <v>2020</v>
       </c>
       <c r="D246" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="E246" t="s">
         <v>256</v>
@@ -11474,13 +11721,13 @@
         <v>2020</v>
       </c>
       <c r="D247" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="E247">
         <v>1132</v>
       </c>
       <c r="F247" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="G247" t="s">
         <v>262</v>
@@ -11507,7 +11754,7 @@
         <v>2020</v>
       </c>
       <c r="D248" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="E248">
         <v>7205</v>
@@ -11516,19 +11763,19 @@
         <v>266</v>
       </c>
       <c r="G248" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
       <c r="H248" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="I248" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="L248" t="b">
         <v>1</v>
       </c>
       <c r="M248" s="5" t="s">
-        <v>982</v>
+        <v>977</v>
       </c>
     </row>
     <row r="249" spans="1:13" x14ac:dyDescent="0.2">
@@ -11542,7 +11789,7 @@
         <v>2020</v>
       </c>
       <c r="D249" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="E249" t="s">
         <v>269</v>
@@ -11575,13 +11822,13 @@
         <v>2020</v>
       </c>
       <c r="D250" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="E250">
         <v>1130</v>
       </c>
       <c r="F250" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="G250" t="s">
         <v>276</v>
@@ -11608,7 +11855,7 @@
         <v>2020</v>
       </c>
       <c r="D251" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="E251">
         <v>244</v>
@@ -11635,25 +11882,25 @@
         <v>46</v>
       </c>
       <c r="B252" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="C252">
         <v>2020</v>
       </c>
       <c r="D252" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="E252">
         <v>1399</v>
       </c>
       <c r="F252" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="G252" t="s">
+        <v>854</v>
+      </c>
+      <c r="I252" t="s">
         <v>855</v>
-      </c>
-      <c r="I252" t="s">
-        <v>856</v>
       </c>
       <c r="J252" t="b">
         <v>1</v>
@@ -11668,25 +11915,25 @@
         <v>47</v>
       </c>
       <c r="B253" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="C253">
         <v>2020</v>
       </c>
       <c r="D253" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="E253">
         <v>245</v>
       </c>
       <c r="F253" t="s">
+        <v>944</v>
+      </c>
+      <c r="G253" t="s">
         <v>945</v>
       </c>
-      <c r="G253" t="s">
+      <c r="I253" t="s">
         <v>946</v>
-      </c>
-      <c r="I253" t="s">
-        <v>947</v>
       </c>
       <c r="J253" t="b">
         <v>1</v>
@@ -11707,7 +11954,7 @@
         <v>2020</v>
       </c>
       <c r="D254" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="E254">
         <v>380</v>
@@ -11740,7 +11987,7 @@
         <v>2020</v>
       </c>
       <c r="D255" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="E255">
         <v>6389</v>
@@ -11773,7 +12020,7 @@
         <v>2020</v>
       </c>
       <c r="D256" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="E256" t="s">
         <v>296</v>
@@ -11806,7 +12053,7 @@
         <v>2020</v>
       </c>
       <c r="D257" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="E257" t="s">
         <v>340</v>
@@ -11839,7 +12086,7 @@
         <v>2020</v>
       </c>
       <c r="D258" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="E258">
         <v>1148</v>
@@ -11872,7 +12119,7 @@
         <v>2020</v>
       </c>
       <c r="D259" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="E259">
         <v>3460</v>
@@ -11905,7 +12152,7 @@
         <v>2020</v>
       </c>
       <c r="D260" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="E260">
         <v>3468</v>
@@ -11938,13 +12185,13 @@
         <v>2020</v>
       </c>
       <c r="D261" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="E261">
         <v>459</v>
       </c>
       <c r="F261" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="G261" t="s">
         <v>148</v>
@@ -11971,7 +12218,7 @@
         <v>2020</v>
       </c>
       <c r="D262" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="E262">
         <v>19073</v>
@@ -12004,13 +12251,13 @@
         <v>2020</v>
       </c>
       <c r="D263" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="E263">
         <v>7233</v>
       </c>
       <c r="F263" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="G263" t="s">
         <v>383</v>
@@ -12037,19 +12284,19 @@
         <v>2020</v>
       </c>
       <c r="D264" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="E264">
         <v>344</v>
       </c>
       <c r="F264" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="G264" t="s">
+        <v>911</v>
+      </c>
+      <c r="I264" t="s">
         <v>912</v>
-      </c>
-      <c r="I264" t="s">
-        <v>913</v>
       </c>
       <c r="J264" t="b">
         <v>1</v>
@@ -12070,7 +12317,7 @@
         <v>2020</v>
       </c>
       <c r="D265" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="E265" t="s">
         <v>662</v>
@@ -12103,7 +12350,7 @@
         <v>2020</v>
       </c>
       <c r="D266" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="E266">
         <v>1131</v>
@@ -12136,22 +12383,22 @@
         <v>2020</v>
       </c>
       <c r="D267" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="E267">
         <v>7232</v>
       </c>
       <c r="F267" t="s">
+        <v>840</v>
+      </c>
+      <c r="G267" t="s">
         <v>841</v>
-      </c>
-      <c r="G267" t="s">
-        <v>842</v>
       </c>
       <c r="H267" t="s">
         <v>495</v>
       </c>
       <c r="I267" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="L267" t="b">
         <v>1</v>
@@ -12169,7 +12416,7 @@
         <v>2020</v>
       </c>
       <c r="D268" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="E268" t="s">
         <v>405</v>
@@ -12202,7 +12449,7 @@
         <v>2020</v>
       </c>
       <c r="D269" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="E269">
         <v>5967</v>
@@ -12235,7 +12482,7 @@
         <v>2020</v>
       </c>
       <c r="D270" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="E270">
         <v>134</v>
@@ -12262,19 +12509,19 @@
         <v>65</v>
       </c>
       <c r="B271" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="C271">
         <v>2020</v>
       </c>
       <c r="D271" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="E271">
         <v>244</v>
       </c>
       <c r="F271" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="G271" t="s">
         <v>281</v>
@@ -12301,7 +12548,7 @@
         <v>2020</v>
       </c>
       <c r="D272" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="E272">
         <v>379</v>
@@ -12334,7 +12581,7 @@
         <v>2020</v>
       </c>
       <c r="D273" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="E273">
         <v>6334</v>
@@ -12367,7 +12614,7 @@
         <v>2020</v>
       </c>
       <c r="D274" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="E274" t="s">
         <v>431</v>

</xml_diff>

<commit_message>
deploymentVerification run 10-23-2024 and lots of fiddling with 2024 verification
</commit_message>
<xml_diff>
--- a/assetManagement/reportOuts/fuzzyMatches_HITL_20241003.xlsx
+++ b/assetManagement/reportOuts/fuzzyMatches_HITL_20241003.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joeduprey/repos/metadataVerification/assetManagement/reportOuts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BD7F846A-0BB6-9440-AD85-89B87356E59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{2BFC7E49-A102-DD49-8E1B-FC5C8A64CFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="760" windowWidth="33120" windowHeight="19740" xr2:uid="{D3F55A4A-1B46-8740-A2A9-3D1205BC3408}"/>
+    <workbookView xWindow="-37980" yWindow="-11120" windowWidth="36960" windowHeight="19260" xr2:uid="{D3F55A4A-1B46-8740-A2A9-3D1205BC3408}"/>
   </bookViews>
   <sheets>
     <sheet name="fuzzyMatches_HITL_20241003" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="1432" uniqueCount="1017">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="1704" uniqueCount="1142">
   <si>
     <t>referenceDesignator</t>
   </si>
@@ -3076,13 +3076,388 @@
   </si>
   <si>
     <t>['ATAPL-78520-00004']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ03C/RASFLA301/RASFLA301_2024/RASFLA301_20240829_115320_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>12881-01</t>
+  </si>
+  <si>
+    <t>['ATAPL-58340-00001']</t>
+  </si>
+  <si>
+    <t>['12881-01']</t>
+  </si>
+  <si>
+    <t>mages/Equipment_Photos/VISIONS24/MJ03C/PPSDNA301/PPSDNA301_2024/PPSDNA301_20240829_115438_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>13003-01</t>
+  </si>
+  <si>
+    <t>['ATAPL-58338-00002']</t>
+  </si>
+  <si>
+    <t>['13003-01']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ03C/CAMDSB303/CAMDSB303_2024/CAMDSB303_20240812_120025_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>19008/19032/19033</t>
+  </si>
+  <si>
+    <t>ATAPL-78437-00008</t>
+  </si>
+  <si>
+    <t>['ATAPL-78437-00008']</t>
+  </si>
+  <si>
+    <t>[0.56, 0.5, 0.5]</t>
+  </si>
+  <si>
+    <t>['SUBC19008', ' SUBC19032', ' SUBC19033']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF03A/SF03A_2024/PCO2WA301_2024/PCO2WA301_20240811_113247_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>[0.75, 0.75, 0.6, 0.5, 0.3]</t>
+  </si>
+  <si>
+    <t>['1248', '1249', 'C0124', ' 61247', ' AQD-12469']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF03A/SF03A_2024/VELPTD302_2024/VELPTD302_20240811_113133_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF03A/SF03A_2024/PHSENA301_2024/PHSENA301_20240811_113534_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>[0.3, 0.38, 0.75, 0.6]</t>
+  </si>
+  <si>
+    <t>[' SUBC20112', '16-50112', '1129', 'P0112']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF03A/SF03A_2024/DOFSTA302_2024/DOFSTA302_20240811_113834_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC03A/PC03A_2024/PHSENA302_2024/20240810_185108.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC03A/PC03A_2024/DOSTAD303_2024/DOSTAD303_20240811_110456_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC03A/PC03A_2024/HYDBBA303_2024/20240810_184952.JPG</t>
+  </si>
+  <si>
+    <t>['1273']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC03A/PC03A_2024/CAMDSC302_2024/CAMDSC302_20240811_110805_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>18827/18831</t>
+  </si>
+  <si>
+    <t>ATAPL-78437-00002</t>
+  </si>
+  <si>
+    <t>['ATAPL-78437-00002']</t>
+  </si>
+  <si>
+    <t>[0.5, 0.56]</t>
+  </si>
+  <si>
+    <t>[' SUBC18827', 'SUBC18831']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LJ03A/DOSTAD301/DOSTAD301_2024/DOSTAD301_20240829_200443_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PN3B/CAMHDA301_2023/CAMHDA301/CAMHDA301_2024/CAMHDA301_20240811_192823_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-70168-0000</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ03B/OSMOIA301/OSMOIA301_2024/OSMOIA301_20240811_193403_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01B/CAMDSB103/CAMDSB103_2024/CAMDSB103_20240820_190026_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>20149/20119</t>
+  </si>
+  <si>
+    <t>ATAPL-78437-00012</t>
+  </si>
+  <si>
+    <t>['ATAPL-78437-00012']</t>
+  </si>
+  <si>
+    <t>[' SUBC20149', 'SUBC20119']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01B/FLOBNM101/FLOBNM101_2024/FLOBNM101_20240820_091940_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01B/FLOBNC101/FLOBNC101_2024/FLOBNC101_20240820_092049_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-58334-00002</t>
+  </si>
+  <si>
+    <t>RS01SUM1-LJ01B-12-VEL3DB104</t>
+  </si>
+  <si>
+    <t>RS01SLBS-MJ01A-12-VEL3DB101</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01A/VEL3DB101/VEL3DB101_2024/VEL3DB101_20240809_125828_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-67979-00006</t>
+  </si>
+  <si>
+    <t>['ATAPL-67979-00006']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01A/DOSTAD101/DOSTAD101_2024/DOSTAD101_20240814_091052_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>['475']</t>
+  </si>
+  <si>
+    <t>RS01SLBS-LJ01A-05-HPIESA101</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01A/HPIESA101/HPIESA101_2024/HPIESA101_20240814_131951_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01A/SF01A_2024/PCO2WA101_2024/PCO2WA101_20240809_074852_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01A/SF01A_2024/VELPTD102_2024/VELPTD102_20240809_074756_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01A/SF01A_2024/PHSENA101_2024/PHSENA101_20240809_074442_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>P0154</t>
+  </si>
+  <si>
+    <t>ATOSU-58337-00012</t>
+  </si>
+  <si>
+    <t>['ATOSU-58337-00012']</t>
+  </si>
+  <si>
+    <t>['P0154']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01A/SF01A_2024/DOFSTA102_2024/DOFSTA102_202</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01A/PC01A_2024/PHSENA102_2024/PHSENA102_20240808_215505_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01A/PC01A_2024/DOSTAD103_2024/DOSTAD103_20240808_215809_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-58320-0000</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01A/PC01A_2024/HYDBBA103_2024/HYDBBA103_20240808_215350_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-58324-00004</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01A/PC01A_2024/CAMDSC102_2024/CAMDSC102_20240808_220032_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>18901/18825</t>
+  </si>
+  <si>
+    <t>['ATAPL-78437-00001']</t>
+  </si>
+  <si>
+    <t>[' SUBC18901', ' SUBC18825']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01B/SF01B_2024/PCO2WA102_2024/PCO2WA102_20240808_151814_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-58336-00008</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01B/SF01B_2024/VELPTD106_2024/VELPTD106_20240808_153315_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>['16P71179-7205', 'AQS-7205']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01B/SF01B_2024/PHSENA108_2024/PHSENA108_20240808_152653_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/SF01B/SF01B_2024/DOFSTA107_2024/DOFSTA107_20240808_153214_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>43-3136</t>
+  </si>
+  <si>
+    <t>['ATOSU-58694-00007']</t>
+  </si>
+  <si>
+    <t>['43-3136']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01B/PC01B_2024/PCO2WA105_2024/PCO2WA105_20240808_144328_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01B/PC01B_2024/PHSENA106_2024/PHSENA106_20240808_143832_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/PC01B/PC01B_2024/ZPLSCB102_2024/ZPLSCB102_20240808_144603_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>4/189</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01C/CAMDSB106/CAMDSB106_2024/CAMDSB106_20240819_160431_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>20161/20145</t>
+  </si>
+  <si>
+    <t>['ATAPL-78437-00013']</t>
+  </si>
+  <si>
+    <t>[' SUBC20161', ' SUBC20145']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01C/LJ01C/LJ01C_2024/HYDBBA105_2024/HYDBBA105_20240818_215805_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-58324-00015</t>
+  </si>
+  <si>
+    <t>['ATOSU-58324-00015']</t>
+  </si>
+  <si>
+    <t>['1249']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01C/LJ01C/LJ01C_2024/PHSEND107_2024/PHSEND107_202</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01C/LJ01C/LJ01C_2024/PCO2WB104_2024/PCO2WB104_2</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01C/LJ01C/LJ01C_2024/VEL3DC107_2024/VEL3DC107_20240818_220312_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/LV01C/LJ01C/LJ01C_2024/DOSTAD108_2024/DOSTAD108_20240818_220219_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>CE02SHBP-MJ01C-08-CAMDSB107</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/CAMDSB107_2024/CAMDSB107_20240815_161937_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>20159/20160</t>
+  </si>
+  <si>
+    <t>['ATAPL-78437-00010']</t>
+  </si>
+  <si>
+    <t>[' SUBC20159', ' SUBC20160']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/ZPLSCB101_2024/ZPLSCB101_20240817_135309_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>190/222</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/LJ01D_2024/HYDBBA106_2024/HYDBBA106_20240817_133234_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>[0.2, 0.15, 0.29, 0.67, 0.5, 0.67, 0.17, 0.4, 0.5]</t>
+  </si>
+  <si>
+    <t>[' SUBC19048', '16P71879-7248', '43-2484', '487', '1248', '248', '5471540-0048', '23248', '1148']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/LJ01D_2024/PHSEND103_2024</t>
+  </si>
+  <si>
+    <t>P0159</t>
+  </si>
+  <si>
+    <t>ATOSU-70571-00004</t>
+  </si>
+  <si>
+    <t>['ATOSU-70571-00004']</t>
+  </si>
+  <si>
+    <t>['P0159']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/LJ01D_2024/PCO2WB103_2024/20240817_133436.JPG</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/LJ01D_2024/VEL3DC108_2024/VEL3DC108_20240817_133850_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-69829-00003</t>
+  </si>
+  <si>
+    <t>[0.44]</t>
+  </si>
+  <si>
+    <t>[' VEC-8167']</t>
+  </si>
+  <si>
+    <t>Images/Equipment_Photos/VISIONS24/MJ01C/LJ01D_2024/DOSTAD106_2024/DOSTAD106_20240817_133101_predeploy.JPG</t>
+  </si>
+  <si>
+    <t>ATAPL-58320-00020</t>
+  </si>
+  <si>
+    <t>[ 'ATAPL-58336-00010']</t>
+  </si>
+  <si>
+    <t>['ATAPL-58337-00002'']</t>
+  </si>
+  <si>
+    <t>no SN for camHD</t>
+  </si>
+  <si>
+    <t>false match need to change script logic to check that it is the same instrument for short SN</t>
+  </si>
+  <si>
+    <t>['ATAPL-70114-00006']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">look at pics again </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ['ATOSU-58324-00014']</t>
+  </si>
+  <si>
+    <t>TODO fix short SN matching</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3217,8 +3592,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="8" tint="0.59999389629810485"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="37">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3422,6 +3804,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -3583,7 +3977,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3591,7 +3985,9 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3967,19 +4363,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BE5CD1D-CC85-4C4C-8EFD-84E97E5F7CE7}">
-  <dimension ref="A1:M274"/>
+  <dimension ref="A1:M326"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="31" customWidth="1"/>
     <col min="3" max="3" width="11.83203125" customWidth="1"/>
-    <col min="4" max="4" width="171.33203125" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="23.6640625" customWidth="1"/>
     <col min="7" max="7" width="39" customWidth="1"/>
     <col min="8" max="8" width="21.33203125" customWidth="1"/>
     <col min="9" max="9" width="34.5" customWidth="1"/>
     <col min="10" max="10" width="18.33203125" customWidth="1"/>
-    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="17.33203125" customWidth="1"/>
     <col min="13" max="13" width="25.83203125" customWidth="1"/>
   </cols>
@@ -5929,7 +6325,7 @@
       <c r="L62" t="b">
         <v>1</v>
       </c>
-      <c r="M62" s="3"/>
+      <c r="M62" s="7"/>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63">
@@ -5959,7 +6355,7 @@
       <c r="L63" t="b">
         <v>1</v>
       </c>
-      <c r="M63" s="3"/>
+      <c r="M63" s="7"/>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64">
@@ -6009,7 +6405,7 @@
       <c r="L65" t="b">
         <v>1</v>
       </c>
-      <c r="M65" s="3"/>
+      <c r="M65" s="7"/>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A66">
@@ -7231,7 +7627,9 @@
       <c r="L104" t="b">
         <v>1</v>
       </c>
-      <c r="M104" s="3"/>
+      <c r="M104" s="7" t="s">
+        <v>1141</v>
+      </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A105">
@@ -7686,7 +8084,7 @@
       <c r="F119" t="s">
         <v>547</v>
       </c>
-      <c r="M119" s="7" t="s">
+      <c r="M119" s="6" t="s">
         <v>1003</v>
       </c>
     </row>
@@ -8903,7 +9301,7 @@
       <c r="L157" t="b">
         <v>1</v>
       </c>
-      <c r="M157" s="3"/>
+      <c r="M157" s="7"/>
     </row>
     <row r="158" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A158">
@@ -8933,7 +9331,7 @@
       <c r="L158" t="b">
         <v>1</v>
       </c>
-      <c r="M158" s="3"/>
+      <c r="M158" s="7"/>
     </row>
     <row r="159" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A159">
@@ -8963,7 +9361,7 @@
       <c r="L159" t="b">
         <v>1</v>
       </c>
-      <c r="M159" s="3"/>
+      <c r="M159" s="7"/>
     </row>
     <row r="160" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A160">
@@ -12370,7 +12768,7 @@
       <c r="L266" t="b">
         <v>1</v>
       </c>
-      <c r="M266" s="3"/>
+      <c r="M266" s="7"/>
     </row>
     <row r="267" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A267">
@@ -12635,6 +13033,1571 @@
         <v>1</v>
       </c>
       <c r="M274" s="3"/>
+    </row>
+    <row r="275" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A275">
+        <v>69</v>
+      </c>
+      <c r="B275" t="s">
+        <v>452</v>
+      </c>
+      <c r="C275">
+        <v>2024</v>
+      </c>
+      <c r="D275" t="s">
+        <v>1017</v>
+      </c>
+      <c r="E275" t="s">
+        <v>1018</v>
+      </c>
+      <c r="G275" t="s">
+        <v>1019</v>
+      </c>
+      <c r="I275" t="s">
+        <v>1020</v>
+      </c>
+      <c r="J275" t="b">
+        <v>1</v>
+      </c>
+      <c r="L275" t="b">
+        <v>1</v>
+      </c>
+      <c r="M275" s="3"/>
+    </row>
+    <row r="276" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A276">
+        <v>70</v>
+      </c>
+      <c r="B276" t="s">
+        <v>448</v>
+      </c>
+      <c r="C276">
+        <v>2024</v>
+      </c>
+      <c r="D276" t="s">
+        <v>1021</v>
+      </c>
+      <c r="E276" t="s">
+        <v>1022</v>
+      </c>
+      <c r="G276" t="s">
+        <v>1023</v>
+      </c>
+      <c r="I276" t="s">
+        <v>1024</v>
+      </c>
+      <c r="J276" t="b">
+        <v>1</v>
+      </c>
+      <c r="L276" t="b">
+        <v>1</v>
+      </c>
+      <c r="M276" s="3"/>
+    </row>
+    <row r="277" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A277">
+        <v>71</v>
+      </c>
+      <c r="B277" t="s">
+        <v>443</v>
+      </c>
+      <c r="C277">
+        <v>2024</v>
+      </c>
+      <c r="D277" t="s">
+        <v>1017</v>
+      </c>
+      <c r="E277" t="s">
+        <v>1018</v>
+      </c>
+      <c r="G277" t="s">
+        <v>1019</v>
+      </c>
+      <c r="I277" t="s">
+        <v>1020</v>
+      </c>
+      <c r="J277" t="b">
+        <v>1</v>
+      </c>
+      <c r="L277" t="b">
+        <v>1</v>
+      </c>
+      <c r="M277" s="3"/>
+    </row>
+    <row r="278" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A278">
+        <v>72</v>
+      </c>
+      <c r="B278" t="s">
+        <v>37</v>
+      </c>
+      <c r="C278">
+        <v>2024</v>
+      </c>
+      <c r="D278" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E278" t="s">
+        <v>1026</v>
+      </c>
+      <c r="F278" t="s">
+        <v>1027</v>
+      </c>
+      <c r="G278" t="s">
+        <v>1028</v>
+      </c>
+      <c r="H278" t="s">
+        <v>1029</v>
+      </c>
+      <c r="I278" t="s">
+        <v>1030</v>
+      </c>
+      <c r="L278" t="b">
+        <v>1</v>
+      </c>
+      <c r="M278" s="3"/>
+    </row>
+    <row r="279" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A279">
+        <v>73</v>
+      </c>
+      <c r="B279" t="s">
+        <v>429</v>
+      </c>
+      <c r="C279">
+        <v>2024</v>
+      </c>
+      <c r="D279" t="s">
+        <v>1031</v>
+      </c>
+      <c r="E279">
+        <v>124</v>
+      </c>
+      <c r="F279" t="s">
+        <v>432</v>
+      </c>
+      <c r="G279" t="s">
+        <v>1134</v>
+      </c>
+      <c r="H279" t="s">
+        <v>1032</v>
+      </c>
+      <c r="I279" t="s">
+        <v>1033</v>
+      </c>
+      <c r="L279" t="b">
+        <v>1</v>
+      </c>
+      <c r="M279" s="3"/>
+    </row>
+    <row r="280" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A280">
+        <v>74</v>
+      </c>
+      <c r="B280" t="s">
+        <v>424</v>
+      </c>
+      <c r="C280">
+        <v>2024</v>
+      </c>
+      <c r="D280" t="s">
+        <v>1034</v>
+      </c>
+      <c r="E280">
+        <v>6334</v>
+      </c>
+      <c r="F280" t="s">
+        <v>426</v>
+      </c>
+      <c r="G280" t="s">
+        <v>427</v>
+      </c>
+      <c r="H280" t="s">
+        <v>292</v>
+      </c>
+      <c r="I280" t="s">
+        <v>428</v>
+      </c>
+      <c r="L280" t="b">
+        <v>1</v>
+      </c>
+      <c r="M280" s="3"/>
+    </row>
+    <row r="281" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A281">
+        <v>75</v>
+      </c>
+      <c r="B281" t="s">
+        <v>403</v>
+      </c>
+      <c r="C281">
+        <v>2024</v>
+      </c>
+      <c r="D281" t="s">
+        <v>1035</v>
+      </c>
+      <c r="E281">
+        <v>112</v>
+      </c>
+      <c r="F281" t="s">
+        <v>406</v>
+      </c>
+      <c r="G281" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H281" t="s">
+        <v>1036</v>
+      </c>
+      <c r="I281" t="s">
+        <v>1037</v>
+      </c>
+      <c r="L281" t="b">
+        <v>1</v>
+      </c>
+      <c r="M281" s="3"/>
+    </row>
+    <row r="282" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A282">
+        <v>76</v>
+      </c>
+      <c r="B282" t="s">
+        <v>401</v>
+      </c>
+      <c r="C282">
+        <v>2024</v>
+      </c>
+      <c r="D282" t="s">
+        <v>1038</v>
+      </c>
+      <c r="F282" t="s">
+        <v>980</v>
+      </c>
+      <c r="G282" t="s">
+        <v>1010</v>
+      </c>
+      <c r="K282" t="b">
+        <v>1</v>
+      </c>
+      <c r="L282" t="b">
+        <v>1</v>
+      </c>
+      <c r="M282" s="3"/>
+    </row>
+    <row r="283" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A283">
+        <v>77</v>
+      </c>
+      <c r="B283" t="s">
+        <v>387</v>
+      </c>
+      <c r="C283">
+        <v>2024</v>
+      </c>
+      <c r="D283" t="s">
+        <v>1039</v>
+      </c>
+      <c r="F283" t="s">
+        <v>390</v>
+      </c>
+      <c r="G283" t="s">
+        <v>391</v>
+      </c>
+      <c r="K283" t="b">
+        <v>1</v>
+      </c>
+      <c r="L283" t="b">
+        <v>1</v>
+      </c>
+      <c r="M283" s="3"/>
+    </row>
+    <row r="284" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A284">
+        <v>78</v>
+      </c>
+      <c r="B284" t="s">
+        <v>385</v>
+      </c>
+      <c r="C284">
+        <v>2024</v>
+      </c>
+      <c r="D284" t="s">
+        <v>1040</v>
+      </c>
+      <c r="F284">
+        <v>5832</v>
+      </c>
+      <c r="M284" s="6" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="285" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A285">
+        <v>79</v>
+      </c>
+      <c r="B285" t="s">
+        <v>376</v>
+      </c>
+      <c r="C285">
+        <v>2024</v>
+      </c>
+      <c r="D285" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E285">
+        <v>1273</v>
+      </c>
+      <c r="F285" t="s">
+        <v>985</v>
+      </c>
+      <c r="G285" t="s">
+        <v>1012</v>
+      </c>
+      <c r="I285" t="s">
+        <v>1042</v>
+      </c>
+      <c r="J285" t="b">
+        <v>1</v>
+      </c>
+      <c r="L285" t="b">
+        <v>1</v>
+      </c>
+      <c r="M285" s="3"/>
+    </row>
+    <row r="286" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A286">
+        <v>80</v>
+      </c>
+      <c r="B286" t="s">
+        <v>373</v>
+      </c>
+      <c r="C286">
+        <v>2024</v>
+      </c>
+      <c r="D286" t="s">
+        <v>1043</v>
+      </c>
+      <c r="E286" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F286" t="s">
+        <v>1045</v>
+      </c>
+      <c r="G286" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H286" t="s">
+        <v>1047</v>
+      </c>
+      <c r="I286" t="s">
+        <v>1048</v>
+      </c>
+      <c r="L286" t="b">
+        <v>1</v>
+      </c>
+      <c r="M286" s="3"/>
+    </row>
+    <row r="287" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A287">
+        <v>81</v>
+      </c>
+      <c r="B287" t="s">
+        <v>334</v>
+      </c>
+      <c r="C287">
+        <v>2024</v>
+      </c>
+      <c r="D287" t="s">
+        <v>1049</v>
+      </c>
+      <c r="E287">
+        <v>273</v>
+      </c>
+      <c r="G287" t="s">
+        <v>336</v>
+      </c>
+      <c r="I287" t="s">
+        <v>337</v>
+      </c>
+      <c r="J287" t="b">
+        <v>1</v>
+      </c>
+      <c r="L287" t="b">
+        <v>1</v>
+      </c>
+      <c r="M287" s="3"/>
+    </row>
+    <row r="288" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A288">
+        <v>82</v>
+      </c>
+      <c r="B288" t="s">
+        <v>34</v>
+      </c>
+      <c r="C288">
+        <v>2024</v>
+      </c>
+      <c r="D288" t="s">
+        <v>1050</v>
+      </c>
+      <c r="F288" t="s">
+        <v>1051</v>
+      </c>
+      <c r="M288" s="4" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="289" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A289">
+        <v>83</v>
+      </c>
+      <c r="B289" t="s">
+        <v>314</v>
+      </c>
+      <c r="C289">
+        <v>2024</v>
+      </c>
+      <c r="D289" t="s">
+        <v>1052</v>
+      </c>
+      <c r="E289">
+        <v>2</v>
+      </c>
+      <c r="G289" t="s">
+        <v>316</v>
+      </c>
+      <c r="I289" t="s">
+        <v>317</v>
+      </c>
+      <c r="J289" t="b">
+        <v>1</v>
+      </c>
+      <c r="L289" t="b">
+        <v>1</v>
+      </c>
+      <c r="M289" s="7" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="290" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A290">
+        <v>84</v>
+      </c>
+      <c r="B290" t="s">
+        <v>311</v>
+      </c>
+      <c r="C290">
+        <v>2024</v>
+      </c>
+      <c r="D290" t="s">
+        <v>1053</v>
+      </c>
+      <c r="E290" t="s">
+        <v>1054</v>
+      </c>
+      <c r="F290" t="s">
+        <v>1055</v>
+      </c>
+      <c r="G290" t="s">
+        <v>1056</v>
+      </c>
+      <c r="H290" t="s">
+        <v>1047</v>
+      </c>
+      <c r="I290" t="s">
+        <v>1057</v>
+      </c>
+      <c r="L290" t="b">
+        <v>1</v>
+      </c>
+      <c r="M290" s="3"/>
+    </row>
+    <row r="291" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A291">
+        <v>85</v>
+      </c>
+      <c r="B291" t="s">
+        <v>307</v>
+      </c>
+      <c r="C291">
+        <v>2024</v>
+      </c>
+      <c r="D291" t="s">
+        <v>1053</v>
+      </c>
+      <c r="E291">
+        <v>1</v>
+      </c>
+      <c r="G291" t="s">
+        <v>309</v>
+      </c>
+      <c r="I291" t="s">
+        <v>310</v>
+      </c>
+      <c r="J291" t="b">
+        <v>1</v>
+      </c>
+      <c r="L291" t="b">
+        <v>1</v>
+      </c>
+      <c r="M291" s="8"/>
+    </row>
+    <row r="292" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A292">
+        <v>86</v>
+      </c>
+      <c r="B292" t="s">
+        <v>303</v>
+      </c>
+      <c r="C292">
+        <v>2024</v>
+      </c>
+      <c r="D292" t="s">
+        <v>1058</v>
+      </c>
+      <c r="E292">
+        <v>3</v>
+      </c>
+      <c r="G292" t="s">
+        <v>305</v>
+      </c>
+      <c r="I292" t="s">
+        <v>306</v>
+      </c>
+      <c r="J292" t="b">
+        <v>1</v>
+      </c>
+      <c r="L292" t="b">
+        <v>1</v>
+      </c>
+      <c r="M292" s="8"/>
+    </row>
+    <row r="293" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A293">
+        <v>87</v>
+      </c>
+      <c r="B293" t="s">
+        <v>300</v>
+      </c>
+      <c r="C293">
+        <v>2024</v>
+      </c>
+      <c r="D293" t="s">
+        <v>1059</v>
+      </c>
+      <c r="E293">
+        <v>2</v>
+      </c>
+      <c r="F293" t="s">
+        <v>1060</v>
+      </c>
+      <c r="G293" t="s">
+        <v>316</v>
+      </c>
+      <c r="I293" t="s">
+        <v>317</v>
+      </c>
+      <c r="J293" t="b">
+        <v>1</v>
+      </c>
+      <c r="L293" t="b">
+        <v>1</v>
+      </c>
+      <c r="M293" s="8"/>
+    </row>
+    <row r="294" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A294">
+        <v>88</v>
+      </c>
+      <c r="B294" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C294">
+        <v>2024</v>
+      </c>
+      <c r="M294" s="6" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="295" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A295">
+        <v>89</v>
+      </c>
+      <c r="B295" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C295">
+        <v>2024</v>
+      </c>
+      <c r="D295" t="s">
+        <v>1063</v>
+      </c>
+      <c r="F295" t="s">
+        <v>1064</v>
+      </c>
+      <c r="G295" t="s">
+        <v>1065</v>
+      </c>
+      <c r="K295" t="b">
+        <v>1</v>
+      </c>
+      <c r="L295" t="b">
+        <v>1</v>
+      </c>
+      <c r="M295" s="3"/>
+    </row>
+    <row r="296" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A296">
+        <v>90</v>
+      </c>
+      <c r="B296" t="s">
+        <v>30</v>
+      </c>
+      <c r="C296">
+        <v>2024</v>
+      </c>
+      <c r="D296" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E296">
+        <v>475</v>
+      </c>
+      <c r="F296" t="s">
+        <v>32</v>
+      </c>
+      <c r="G296" t="s">
+        <v>33</v>
+      </c>
+      <c r="I296" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J296" t="b">
+        <v>1</v>
+      </c>
+      <c r="L296" t="b">
+        <v>1</v>
+      </c>
+      <c r="M296" s="3"/>
+    </row>
+    <row r="297" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A297">
+        <v>91</v>
+      </c>
+      <c r="B297" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C297">
+        <v>2024</v>
+      </c>
+      <c r="D297" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E297">
+        <v>308</v>
+      </c>
+      <c r="G297" t="s">
+        <v>320</v>
+      </c>
+      <c r="H297" t="s">
+        <v>321</v>
+      </c>
+      <c r="I297" t="s">
+        <v>322</v>
+      </c>
+      <c r="L297" t="b">
+        <v>1</v>
+      </c>
+      <c r="M297" s="3"/>
+    </row>
+    <row r="298" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A298">
+        <v>92</v>
+      </c>
+      <c r="B298" t="s">
+        <v>294</v>
+      </c>
+      <c r="C298">
+        <v>2024</v>
+      </c>
+      <c r="D298" t="s">
+        <v>1070</v>
+      </c>
+      <c r="E298" t="s">
+        <v>296</v>
+      </c>
+      <c r="F298" t="s">
+        <v>297</v>
+      </c>
+      <c r="G298" t="s">
+        <v>298</v>
+      </c>
+      <c r="I298" t="s">
+        <v>299</v>
+      </c>
+      <c r="J298" t="b">
+        <v>1</v>
+      </c>
+      <c r="L298" t="b">
+        <v>1</v>
+      </c>
+      <c r="M298" s="3"/>
+    </row>
+    <row r="299" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A299">
+        <v>93</v>
+      </c>
+      <c r="B299" t="s">
+        <v>288</v>
+      </c>
+      <c r="C299">
+        <v>2024</v>
+      </c>
+      <c r="D299" t="s">
+        <v>1071</v>
+      </c>
+      <c r="E299">
+        <v>6389</v>
+      </c>
+      <c r="F299" t="s">
+        <v>290</v>
+      </c>
+      <c r="G299" t="s">
+        <v>291</v>
+      </c>
+      <c r="H299" t="s">
+        <v>292</v>
+      </c>
+      <c r="I299" t="s">
+        <v>293</v>
+      </c>
+      <c r="L299" t="b">
+        <v>1</v>
+      </c>
+      <c r="M299" s="3"/>
+    </row>
+    <row r="300" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A300">
+        <v>94</v>
+      </c>
+      <c r="B300" t="s">
+        <v>267</v>
+      </c>
+      <c r="C300">
+        <v>2024</v>
+      </c>
+      <c r="D300" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E300" t="s">
+        <v>1073</v>
+      </c>
+      <c r="F300" t="s">
+        <v>1074</v>
+      </c>
+      <c r="G300" t="s">
+        <v>1075</v>
+      </c>
+      <c r="I300" t="s">
+        <v>1076</v>
+      </c>
+      <c r="J300" t="b">
+        <v>1</v>
+      </c>
+      <c r="L300" t="b">
+        <v>1</v>
+      </c>
+      <c r="M300" s="3"/>
+    </row>
+    <row r="301" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A301">
+        <v>95</v>
+      </c>
+      <c r="B301" t="s">
+        <v>656</v>
+      </c>
+      <c r="C301">
+        <v>2024</v>
+      </c>
+      <c r="D301" t="s">
+        <v>1077</v>
+      </c>
+      <c r="F301" t="s">
+        <v>174</v>
+      </c>
+      <c r="G301" t="s">
+        <v>175</v>
+      </c>
+      <c r="K301" t="b">
+        <v>1</v>
+      </c>
+      <c r="L301" t="b">
+        <v>1</v>
+      </c>
+      <c r="M301" s="3"/>
+    </row>
+    <row r="302" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A302">
+        <v>96</v>
+      </c>
+      <c r="B302" t="s">
+        <v>254</v>
+      </c>
+      <c r="C302">
+        <v>2024</v>
+      </c>
+      <c r="D302" t="s">
+        <v>1078</v>
+      </c>
+      <c r="E302" t="s">
+        <v>256</v>
+      </c>
+      <c r="F302" t="s">
+        <v>257</v>
+      </c>
+      <c r="G302" t="s">
+        <v>258</v>
+      </c>
+      <c r="I302" t="s">
+        <v>259</v>
+      </c>
+      <c r="J302" t="b">
+        <v>1</v>
+      </c>
+      <c r="L302" t="b">
+        <v>1</v>
+      </c>
+      <c r="M302" s="3"/>
+    </row>
+    <row r="303" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A303">
+        <v>97</v>
+      </c>
+      <c r="B303" t="s">
+        <v>638</v>
+      </c>
+      <c r="C303">
+        <v>2024</v>
+      </c>
+      <c r="D303" t="s">
+        <v>1079</v>
+      </c>
+      <c r="F303" t="s">
+        <v>1080</v>
+      </c>
+      <c r="M303" s="6" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="304" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A304">
+        <v>98</v>
+      </c>
+      <c r="B304" t="s">
+        <v>244</v>
+      </c>
+      <c r="C304">
+        <v>2024</v>
+      </c>
+      <c r="D304" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E304">
+        <v>1272</v>
+      </c>
+      <c r="F304" t="s">
+        <v>1082</v>
+      </c>
+      <c r="G304" t="s">
+        <v>378</v>
+      </c>
+      <c r="I304" t="s">
+        <v>379</v>
+      </c>
+      <c r="J304" t="b">
+        <v>1</v>
+      </c>
+      <c r="L304" t="b">
+        <v>1</v>
+      </c>
+      <c r="M304" s="3"/>
+    </row>
+    <row r="305" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A305">
+        <v>99</v>
+      </c>
+      <c r="B305" t="s">
+        <v>241</v>
+      </c>
+      <c r="C305">
+        <v>2024</v>
+      </c>
+      <c r="D305" t="s">
+        <v>1083</v>
+      </c>
+      <c r="E305" t="s">
+        <v>1084</v>
+      </c>
+      <c r="F305" t="s">
+        <v>375</v>
+      </c>
+      <c r="G305" t="s">
+        <v>1085</v>
+      </c>
+      <c r="H305" t="s">
+        <v>505</v>
+      </c>
+      <c r="I305" t="s">
+        <v>1086</v>
+      </c>
+      <c r="L305" t="b">
+        <v>1</v>
+      </c>
+      <c r="M305" s="3"/>
+    </row>
+    <row r="306" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A306">
+        <v>100</v>
+      </c>
+      <c r="B306" t="s">
+        <v>202</v>
+      </c>
+      <c r="C306">
+        <v>2024</v>
+      </c>
+      <c r="D306" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E306" t="s">
+        <v>204</v>
+      </c>
+      <c r="F306" t="s">
+        <v>1088</v>
+      </c>
+      <c r="G306" t="s">
+        <v>206</v>
+      </c>
+      <c r="I306" t="s">
+        <v>207</v>
+      </c>
+      <c r="J306" t="b">
+        <v>1</v>
+      </c>
+      <c r="L306" t="b">
+        <v>1</v>
+      </c>
+      <c r="M306" s="3"/>
+    </row>
+    <row r="307" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A307">
+        <v>101</v>
+      </c>
+      <c r="B307" t="s">
+        <v>197</v>
+      </c>
+      <c r="C307">
+        <v>2024</v>
+      </c>
+      <c r="D307" t="s">
+        <v>1089</v>
+      </c>
+      <c r="E307">
+        <v>7205</v>
+      </c>
+      <c r="F307" t="s">
+        <v>200</v>
+      </c>
+      <c r="G307" t="s">
+        <v>1138</v>
+      </c>
+      <c r="H307" t="s">
+        <v>936</v>
+      </c>
+      <c r="I307" t="s">
+        <v>1090</v>
+      </c>
+      <c r="L307" t="b">
+        <v>1</v>
+      </c>
+      <c r="M307" s="3"/>
+    </row>
+    <row r="308" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A308">
+        <v>102</v>
+      </c>
+      <c r="B308" t="s">
+        <v>176</v>
+      </c>
+      <c r="C308">
+        <v>2024</v>
+      </c>
+      <c r="D308" t="s">
+        <v>1091</v>
+      </c>
+      <c r="E308" t="s">
+        <v>178</v>
+      </c>
+      <c r="F308" t="s">
+        <v>179</v>
+      </c>
+      <c r="G308" t="s">
+        <v>180</v>
+      </c>
+      <c r="I308" t="s">
+        <v>181</v>
+      </c>
+      <c r="J308" t="b">
+        <v>1</v>
+      </c>
+      <c r="L308" t="b">
+        <v>1</v>
+      </c>
+      <c r="M308" s="3"/>
+    </row>
+    <row r="309" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A309">
+        <v>103</v>
+      </c>
+      <c r="B309" t="s">
+        <v>172</v>
+      </c>
+      <c r="C309">
+        <v>2024</v>
+      </c>
+      <c r="D309" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E309" t="s">
+        <v>1093</v>
+      </c>
+      <c r="G309" t="s">
+        <v>1094</v>
+      </c>
+      <c r="I309" t="s">
+        <v>1095</v>
+      </c>
+      <c r="J309" t="b">
+        <v>1</v>
+      </c>
+      <c r="L309" t="b">
+        <v>1</v>
+      </c>
+      <c r="M309" s="3"/>
+    </row>
+    <row r="310" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A310">
+        <v>104</v>
+      </c>
+      <c r="B310" t="s">
+        <v>162</v>
+      </c>
+      <c r="C310">
+        <v>2024</v>
+      </c>
+      <c r="D310" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E310" t="s">
+        <v>164</v>
+      </c>
+      <c r="F310" t="s">
+        <v>165</v>
+      </c>
+      <c r="G310" t="s">
+        <v>166</v>
+      </c>
+      <c r="I310" t="s">
+        <v>167</v>
+      </c>
+      <c r="J310" t="b">
+        <v>1</v>
+      </c>
+      <c r="L310" t="b">
+        <v>1</v>
+      </c>
+      <c r="M310" s="3"/>
+    </row>
+    <row r="311" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A311">
+        <v>105</v>
+      </c>
+      <c r="B311" t="s">
+        <v>156</v>
+      </c>
+      <c r="C311">
+        <v>2024</v>
+      </c>
+      <c r="D311" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E311" t="s">
+        <v>158</v>
+      </c>
+      <c r="F311" t="s">
+        <v>159</v>
+      </c>
+      <c r="G311" t="s">
+        <v>160</v>
+      </c>
+      <c r="I311" t="s">
+        <v>161</v>
+      </c>
+      <c r="J311" t="b">
+        <v>1</v>
+      </c>
+      <c r="L311" t="b">
+        <v>1</v>
+      </c>
+      <c r="M311" s="3"/>
+    </row>
+    <row r="312" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A312">
+        <v>106</v>
+      </c>
+      <c r="B312" t="s">
+        <v>553</v>
+      </c>
+      <c r="C312">
+        <v>2024</v>
+      </c>
+      <c r="M312" s="6" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="313" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A313">
+        <v>107</v>
+      </c>
+      <c r="B313" t="s">
+        <v>545</v>
+      </c>
+      <c r="C313">
+        <v>2024</v>
+      </c>
+      <c r="D313" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E313" t="s">
+        <v>1099</v>
+      </c>
+      <c r="G313" t="s">
+        <v>705</v>
+      </c>
+      <c r="I313" t="s">
+        <v>706</v>
+      </c>
+      <c r="J313" t="b">
+        <v>1</v>
+      </c>
+      <c r="L313" t="b">
+        <v>1</v>
+      </c>
+      <c r="M313" s="8"/>
+    </row>
+    <row r="314" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A314">
+        <v>108</v>
+      </c>
+      <c r="B314" t="s">
+        <v>126</v>
+      </c>
+      <c r="C314">
+        <v>2024</v>
+      </c>
+      <c r="D314" t="s">
+        <v>1100</v>
+      </c>
+      <c r="E314" t="s">
+        <v>1101</v>
+      </c>
+      <c r="G314" t="s">
+        <v>1102</v>
+      </c>
+      <c r="H314" t="s">
+        <v>505</v>
+      </c>
+      <c r="I314" t="s">
+        <v>1103</v>
+      </c>
+      <c r="L314" t="b">
+        <v>1</v>
+      </c>
+      <c r="M314" s="3"/>
+    </row>
+    <row r="315" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A315">
+        <v>109</v>
+      </c>
+      <c r="B315" t="s">
+        <v>124</v>
+      </c>
+      <c r="C315">
+        <v>2024</v>
+      </c>
+      <c r="D315" t="s">
+        <v>1104</v>
+      </c>
+      <c r="E315">
+        <v>1249</v>
+      </c>
+      <c r="F315" t="s">
+        <v>1105</v>
+      </c>
+      <c r="G315" t="s">
+        <v>1106</v>
+      </c>
+      <c r="I315" t="s">
+        <v>1107</v>
+      </c>
+      <c r="J315" t="b">
+        <v>1</v>
+      </c>
+      <c r="L315" t="b">
+        <v>1</v>
+      </c>
+      <c r="M315" s="3"/>
+    </row>
+    <row r="316" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A316">
+        <v>110</v>
+      </c>
+      <c r="B316" t="s">
+        <v>118</v>
+      </c>
+      <c r="C316">
+        <v>2024</v>
+      </c>
+      <c r="D316" t="s">
+        <v>1108</v>
+      </c>
+      <c r="E316" t="s">
+        <v>120</v>
+      </c>
+      <c r="F316" t="s">
+        <v>121</v>
+      </c>
+      <c r="G316" t="s">
+        <v>122</v>
+      </c>
+      <c r="I316" t="s">
+        <v>123</v>
+      </c>
+      <c r="J316" t="b">
+        <v>1</v>
+      </c>
+      <c r="L316" t="b">
+        <v>1</v>
+      </c>
+      <c r="M316" s="3"/>
+    </row>
+    <row r="317" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A317">
+        <v>111</v>
+      </c>
+      <c r="B317" t="s">
+        <v>112</v>
+      </c>
+      <c r="C317">
+        <v>2024</v>
+      </c>
+      <c r="D317" t="s">
+        <v>1109</v>
+      </c>
+      <c r="E317" t="s">
+        <v>114</v>
+      </c>
+      <c r="F317" t="s">
+        <v>115</v>
+      </c>
+      <c r="G317" t="s">
+        <v>116</v>
+      </c>
+      <c r="I317" t="s">
+        <v>117</v>
+      </c>
+      <c r="J317" t="b">
+        <v>1</v>
+      </c>
+      <c r="L317" t="b">
+        <v>1</v>
+      </c>
+      <c r="M317" s="3"/>
+    </row>
+    <row r="318" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A318">
+        <v>112</v>
+      </c>
+      <c r="B318" t="s">
+        <v>101</v>
+      </c>
+      <c r="C318">
+        <v>2024</v>
+      </c>
+      <c r="D318" t="s">
+        <v>1110</v>
+      </c>
+      <c r="E318" t="s">
+        <v>103</v>
+      </c>
+      <c r="F318" t="s">
+        <v>104</v>
+      </c>
+      <c r="G318" t="s">
+        <v>105</v>
+      </c>
+      <c r="H318" t="s">
+        <v>61</v>
+      </c>
+      <c r="I318" t="s">
+        <v>106</v>
+      </c>
+      <c r="L318" t="b">
+        <v>1</v>
+      </c>
+      <c r="M318" s="3"/>
+    </row>
+    <row r="319" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A319">
+        <v>113</v>
+      </c>
+      <c r="B319" t="s">
+        <v>96</v>
+      </c>
+      <c r="C319">
+        <v>2024</v>
+      </c>
+      <c r="D319" t="s">
+        <v>1111</v>
+      </c>
+      <c r="E319">
+        <v>133</v>
+      </c>
+      <c r="F319" t="s">
+        <v>98</v>
+      </c>
+      <c r="G319" t="s">
+        <v>99</v>
+      </c>
+      <c r="I319" t="s">
+        <v>100</v>
+      </c>
+      <c r="J319" t="b">
+        <v>1</v>
+      </c>
+      <c r="L319" t="b">
+        <v>1</v>
+      </c>
+      <c r="M319" s="3"/>
+    </row>
+    <row r="320" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A320">
+        <v>114</v>
+      </c>
+      <c r="B320" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C320">
+        <v>2024</v>
+      </c>
+      <c r="D320" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E320" t="s">
+        <v>1114</v>
+      </c>
+      <c r="G320" t="s">
+        <v>1115</v>
+      </c>
+      <c r="H320" t="s">
+        <v>505</v>
+      </c>
+      <c r="I320" t="s">
+        <v>1116</v>
+      </c>
+      <c r="L320" t="b">
+        <v>1</v>
+      </c>
+      <c r="M320" s="3"/>
+    </row>
+    <row r="321" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A321">
+        <v>115</v>
+      </c>
+      <c r="B321" t="s">
+        <v>84</v>
+      </c>
+      <c r="C321">
+        <v>2024</v>
+      </c>
+      <c r="D321" t="s">
+        <v>1117</v>
+      </c>
+      <c r="E321" t="s">
+        <v>1118</v>
+      </c>
+      <c r="M321" s="9" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="322" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A322">
+        <v>116</v>
+      </c>
+      <c r="B322" t="s">
+        <v>80</v>
+      </c>
+      <c r="C322">
+        <v>2024</v>
+      </c>
+      <c r="D322" t="s">
+        <v>1119</v>
+      </c>
+      <c r="E322">
+        <v>48</v>
+      </c>
+      <c r="G322" t="s">
+        <v>1140</v>
+      </c>
+      <c r="H322" t="s">
+        <v>1120</v>
+      </c>
+      <c r="I322" t="s">
+        <v>1121</v>
+      </c>
+      <c r="L322" t="b">
+        <v>1</v>
+      </c>
+      <c r="M322" s="3"/>
+    </row>
+    <row r="323" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A323">
+        <v>117</v>
+      </c>
+      <c r="B323" t="s">
+        <v>74</v>
+      </c>
+      <c r="C323">
+        <v>2024</v>
+      </c>
+      <c r="D323" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E323" t="s">
+        <v>1123</v>
+      </c>
+      <c r="F323" t="s">
+        <v>1124</v>
+      </c>
+      <c r="G323" t="s">
+        <v>1125</v>
+      </c>
+      <c r="I323" t="s">
+        <v>1126</v>
+      </c>
+      <c r="J323" t="b">
+        <v>1</v>
+      </c>
+      <c r="L323" t="b">
+        <v>1</v>
+      </c>
+      <c r="M323" s="3"/>
+    </row>
+    <row r="324" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A324">
+        <v>118</v>
+      </c>
+      <c r="B324" t="s">
+        <v>68</v>
+      </c>
+      <c r="C324">
+        <v>2024</v>
+      </c>
+      <c r="D324" t="s">
+        <v>1127</v>
+      </c>
+      <c r="E324" t="s">
+        <v>70</v>
+      </c>
+      <c r="F324" t="s">
+        <v>71</v>
+      </c>
+      <c r="G324" t="s">
+        <v>72</v>
+      </c>
+      <c r="I324" t="s">
+        <v>73</v>
+      </c>
+      <c r="J324" t="b">
+        <v>1</v>
+      </c>
+      <c r="L324" t="b">
+        <v>1</v>
+      </c>
+      <c r="M324" s="3"/>
+    </row>
+    <row r="325" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A325">
+        <v>119</v>
+      </c>
+      <c r="B325" t="s">
+        <v>56</v>
+      </c>
+      <c r="C325">
+        <v>2024</v>
+      </c>
+      <c r="D325" t="s">
+        <v>1128</v>
+      </c>
+      <c r="E325">
+        <v>8167</v>
+      </c>
+      <c r="F325" t="s">
+        <v>1129</v>
+      </c>
+      <c r="G325" t="s">
+        <v>60</v>
+      </c>
+      <c r="H325" t="s">
+        <v>1130</v>
+      </c>
+      <c r="I325" t="s">
+        <v>1131</v>
+      </c>
+      <c r="L325" t="b">
+        <v>1</v>
+      </c>
+      <c r="M325" s="3"/>
+    </row>
+    <row r="326" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A326">
+        <v>120</v>
+      </c>
+      <c r="B326" t="s">
+        <v>51</v>
+      </c>
+      <c r="C326">
+        <v>2024</v>
+      </c>
+      <c r="D326" t="s">
+        <v>1132</v>
+      </c>
+      <c r="E326">
+        <v>216</v>
+      </c>
+      <c r="F326" t="s">
+        <v>1133</v>
+      </c>
+      <c r="G326" t="s">
+        <v>54</v>
+      </c>
+      <c r="I326" t="s">
+        <v>55</v>
+      </c>
+      <c r="J326" t="b">
+        <v>1</v>
+      </c>
+      <c r="L326" t="b">
+        <v>1</v>
+      </c>
+      <c r="M326" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>